<commit_message>
Exceptions: Salt Shark Sep extensions, Flo & Frankie cut-off agreement, Vixxen 5 Oct Farmers deadline
Order-Level Exceptions (Order Cut Off, Count as met, logged 2026-10-01):
- Salt Shark 4938 and 4953, month 2026-09 (orders created 29/30 Sep)
- Flo & Frankie '*', open-ended, per customer agreement

Order Content-Based Overrides:
- Vixxen, Delivery Company Name contains 'farmers', Fixed (2026-10-13 20:00),
  effective 2026-10-05 only. All 55 Farmers orders created 5 Oct move from
  6 Oct 17:00 to 13 Oct 20:00; the 6 non-Farmers orders that day were
  already dispatched on time.

Edited with openpyxl on a GitHub Actions runner from latest main and checked
against CartonCloud; other sheets' row counts and charts unchanged. Also
removes the temporary exceptions-check workflow.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/pipeline/kpi_dashboard.xlsx
+++ b/pipeline/kpi_dashboard.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Charts" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPI Schedule" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Customers" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPI_Data" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exceptions" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Issue Log" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard_Calc" sheetId="10" state="hidden" r:id="rId10"/>
+    <sheet name="Instructions" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Dashboard" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Charts" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Read Me" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="KPI Schedule" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Customers" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="KPI_Data" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Exceptions" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Issue Log" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Dashboard_Calc" sheetId="10" state="hidden" r:id="rId10"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'KPI_Data'!$A$3:$J$295</definedName>
@@ -292,7 +292,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="92">
+  <cellXfs count="93">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -559,6 +559,9 @@
     </xf>
     <xf numFmtId="169" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="170" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -695,14 +698,14 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr rot="0"/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -724,8 +727,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -750,10 +753,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:srgbClr val="4A7EBB"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+            <a:ln w="12600">
               <a:solidFill>
                 <a:srgbClr val="4A7EBB"/>
               </a:solidFill>
@@ -764,16 +767,16 @@
           <marker>
             <symbol val="none"/>
             <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:ln>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
           </marker>
           <dLbls>
             <txPr>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr wrap="square"/>
+              <a:lstStyle/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -902,10 +905,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:srgbClr val="BE4B48"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+            <a:ln w="12600">
               <a:solidFill>
                 <a:srgbClr val="BE4B48"/>
               </a:solidFill>
@@ -916,16 +919,16 @@
           <marker>
             <symbol val="none"/>
             <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:ln>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
           </marker>
           <dLbls>
             <txPr>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr wrap="square"/>
+              <a:lstStyle/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -1020,7 +1023,7 @@
         </ser>
         <hiLowLines>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+            <a:ln w="0">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -1042,7 +1045,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+          <a:ln w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -1051,9 +1054,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -1084,7 +1087,7 @@
         <axPos val="l"/>
         <majorGridlines>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+            <a:ln w="9360">
               <a:solidFill>
                 <a:srgbClr val="878787"/>
               </a:solidFill>
@@ -1096,9 +1099,9 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="-5400000"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr rot="-5400000"/>
+              <a:lstStyle/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr sz="1300" b="0" strike="noStrike">
                     <a:uFillTx/>
@@ -1120,8 +1123,8 @@
           </tx>
           <overlay val="0"/>
           <spPr>
-            <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+            <a:noFill/>
+            <a:ln w="0">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -1132,7 +1135,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+          <a:ln w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -1141,9 +1144,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -1167,16 +1170,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -1196,10 +1199,10 @@
     <dispBlanksAs val="zero"/>
   </chart>
   <spPr>
-    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+    <a:solidFill>
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+    <a:ln w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -1211,14 +1214,14 @@
 </file>
 
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr rot="0"/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -1240,8 +1243,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -1266,10 +1269,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:srgbClr val="4A7EBB"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+            <a:ln w="12600">
               <a:solidFill>
                 <a:srgbClr val="4A7EBB"/>
               </a:solidFill>
@@ -1280,16 +1283,16 @@
           <marker>
             <symbol val="none"/>
             <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:ln>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
           </marker>
           <dLbls>
             <txPr>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr wrap="square"/>
+              <a:lstStyle/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -1418,10 +1421,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:srgbClr val="BE4B48"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+            <a:ln w="12600">
               <a:solidFill>
                 <a:srgbClr val="BE4B48"/>
               </a:solidFill>
@@ -1432,16 +1435,16 @@
           <marker>
             <symbol val="none"/>
             <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:ln>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
           </marker>
           <dLbls>
             <txPr>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr wrap="square"/>
+              <a:lstStyle/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -1521,7 +1524,7 @@
         </ser>
         <hiLowLines>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+            <a:ln w="0">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -1543,7 +1546,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+          <a:ln w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -1552,9 +1555,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -1585,7 +1588,7 @@
         <axPos val="l"/>
         <majorGridlines>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+            <a:ln w="9360">
               <a:solidFill>
                 <a:srgbClr val="878787"/>
               </a:solidFill>
@@ -1597,9 +1600,9 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="-5400000"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr rot="-5400000"/>
+              <a:lstStyle/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr sz="1300" b="0" strike="noStrike">
                     <a:uFillTx/>
@@ -1621,8 +1624,8 @@
           </tx>
           <overlay val="0"/>
           <spPr>
-            <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+            <a:noFill/>
+            <a:ln w="0">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -1633,7 +1636,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+          <a:ln w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -1642,9 +1645,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -1668,16 +1671,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -1697,10 +1700,10 @@
     <dispBlanksAs val="zero"/>
   </chart>
   <spPr>
-    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+    <a:solidFill>
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+    <a:ln w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -1712,14 +1715,14 @@
 </file>
 
 <file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr rot="0"/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -1741,8 +1744,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -1767,10 +1770,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:srgbClr val="4A7EBB"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+            <a:ln w="12600">
               <a:solidFill>
                 <a:srgbClr val="4A7EBB"/>
               </a:solidFill>
@@ -1781,16 +1784,16 @@
           <marker>
             <symbol val="none"/>
             <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:ln>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
           </marker>
           <dLbls>
             <txPr>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr wrap="square"/>
+              <a:lstStyle/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -1919,10 +1922,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:srgbClr val="BE4B48"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+            <a:ln w="12600">
               <a:solidFill>
                 <a:srgbClr val="BE4B48"/>
               </a:solidFill>
@@ -1933,16 +1936,16 @@
           <marker>
             <symbol val="none"/>
             <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:ln>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
           </marker>
           <dLbls>
             <txPr>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr wrap="square"/>
+              <a:lstStyle/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -2040,7 +2043,7 @@
         </ser>
         <hiLowLines>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+            <a:ln w="0">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -2062,7 +2065,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+          <a:ln w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2071,9 +2074,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2104,7 +2107,7 @@
         <axPos val="l"/>
         <majorGridlines>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+            <a:ln w="9360">
               <a:solidFill>
                 <a:srgbClr val="878787"/>
               </a:solidFill>
@@ -2116,9 +2119,9 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="-5400000"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr rot="-5400000"/>
+              <a:lstStyle/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr sz="1300" b="0" strike="noStrike">
                     <a:uFillTx/>
@@ -2140,8 +2143,8 @@
           </tx>
           <overlay val="0"/>
           <spPr>
-            <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+            <a:noFill/>
+            <a:ln w="0">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -2152,7 +2155,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+          <a:ln w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2161,9 +2164,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2187,16 +2190,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -2216,10 +2219,10 @@
     <dispBlanksAs val="zero"/>
   </chart>
   <spPr>
-    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+    <a:solidFill>
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+    <a:ln w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -2231,14 +2234,14 @@
 </file>
 
 <file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr rot="0"/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -2260,8 +2263,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -2286,10 +2289,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:srgbClr val="4A7EBB"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+            <a:ln w="12600">
               <a:solidFill>
                 <a:srgbClr val="4A7EBB"/>
               </a:solidFill>
@@ -2300,16 +2303,16 @@
           <marker>
             <symbol val="none"/>
             <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:ln>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
           </marker>
           <dLbls>
             <txPr>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr wrap="square"/>
+              <a:lstStyle/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -2438,10 +2441,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:srgbClr val="BE4B48"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+            <a:ln w="12600">
               <a:solidFill>
                 <a:srgbClr val="BE4B48"/>
               </a:solidFill>
@@ -2452,16 +2455,16 @@
           <marker>
             <symbol val="none"/>
             <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:ln>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
           </marker>
           <dLbls>
             <txPr>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr wrap="square"/>
+              <a:lstStyle/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -2547,7 +2550,7 @@
         </ser>
         <hiLowLines>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+            <a:ln w="0">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -2569,7 +2572,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+          <a:ln w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2578,9 +2581,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2611,7 +2614,7 @@
         <axPos val="l"/>
         <majorGridlines>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+            <a:ln w="9360">
               <a:solidFill>
                 <a:srgbClr val="878787"/>
               </a:solidFill>
@@ -2623,9 +2626,9 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="-5400000"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr rot="-5400000"/>
+              <a:lstStyle/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr sz="1300" b="0" strike="noStrike">
                     <a:uFillTx/>
@@ -2647,8 +2650,8 @@
           </tx>
           <overlay val="0"/>
           <spPr>
-            <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+            <a:noFill/>
+            <a:ln w="0">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -2659,7 +2662,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+          <a:ln w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2668,9 +2671,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2694,16 +2697,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -2723,10 +2726,10 @@
     <dispBlanksAs val="zero"/>
   </chart>
   <spPr>
-    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+    <a:solidFill>
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+    <a:ln w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -2738,14 +2741,14 @@
 </file>
 
 <file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr rot="0"/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -2767,8 +2770,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -2793,10 +2796,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:srgbClr val="4A7EBB"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+            <a:ln w="12600">
               <a:solidFill>
                 <a:srgbClr val="4A7EBB"/>
               </a:solidFill>
@@ -2807,16 +2810,16 @@
           <marker>
             <symbol val="none"/>
             <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:ln>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
           </marker>
           <dLbls>
             <txPr>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr wrap="square"/>
+              <a:lstStyle/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -2945,10 +2948,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:srgbClr val="BE4B48"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+            <a:ln w="12600">
               <a:solidFill>
                 <a:srgbClr val="BE4B48"/>
               </a:solidFill>
@@ -2959,16 +2962,16 @@
           <marker>
             <symbol val="none"/>
             <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:ln>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
           </marker>
           <dLbls>
             <txPr>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr wrap="square"/>
+              <a:lstStyle/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -3057,7 +3060,7 @@
         </ser>
         <hiLowLines>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+            <a:ln w="0">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -3079,7 +3082,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+          <a:ln w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -3088,9 +3091,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -3121,7 +3124,7 @@
         <axPos val="l"/>
         <majorGridlines>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+            <a:ln w="9360">
               <a:solidFill>
                 <a:srgbClr val="878787"/>
               </a:solidFill>
@@ -3133,9 +3136,9 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="-5400000"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr rot="-5400000"/>
+              <a:lstStyle/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr sz="1300" b="0" strike="noStrike">
                     <a:uFillTx/>
@@ -3157,8 +3160,8 @@
           </tx>
           <overlay val="0"/>
           <spPr>
-            <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+            <a:noFill/>
+            <a:ln w="0">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -3169,7 +3172,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+          <a:ln w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -3178,9 +3181,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -3204,16 +3207,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -3233,10 +3236,10 @@
     <dispBlanksAs val="zero"/>
   </chart>
   <spPr>
-    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+    <a:solidFill>
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+    <a:ln w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -3248,14 +3251,14 @@
 </file>
 
 <file path=xl/charts/chart6.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr rot="0"/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -3277,8 +3280,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -3304,10 +3307,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+            <a:ln w="12600">
               <a:solidFill>
                 <a:srgbClr val="F9F9F9"/>
               </a:solidFill>
@@ -3318,9 +3321,9 @@
           <invertIfNegative val="0"/>
           <dLbls>
             <txPr>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr wrap="square"/>
+              <a:lstStyle/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -3388,10 +3391,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:srgbClr val="C0504D"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+            <a:ln w="12600">
               <a:solidFill>
                 <a:srgbClr val="F9F9F9"/>
               </a:solidFill>
@@ -3402,9 +3405,9 @@
           <invertIfNegative val="0"/>
           <dLbls>
             <txPr>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr wrap="square"/>
+              <a:lstStyle/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -3468,7 +3471,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+          <a:ln w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -3477,9 +3480,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -3510,7 +3513,7 @@
         <axPos val="l"/>
         <majorGridlines>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+            <a:ln w="9360">
               <a:solidFill>
                 <a:srgbClr val="878787"/>
               </a:solidFill>
@@ -3524,7 +3527,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+          <a:ln w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -3533,9 +3536,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -3559,16 +3562,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -3588,10 +3591,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+    <a:solidFill>
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+    <a:ln w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -3603,14 +3606,14 @@
 </file>
 
 <file path=xl/charts/chart7.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr rot="0"/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -3632,8 +3635,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -3659,10 +3662,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+            <a:ln w="12600">
               <a:solidFill>
                 <a:srgbClr val="F9F9F9"/>
               </a:solidFill>
@@ -3673,9 +3676,9 @@
           <invertIfNegative val="0"/>
           <dLbls>
             <txPr>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr wrap="square"/>
+              <a:lstStyle/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -3743,10 +3746,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:srgbClr val="C0504D"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+            <a:ln w="12600">
               <a:solidFill>
                 <a:srgbClr val="F9F9F9"/>
               </a:solidFill>
@@ -3757,9 +3760,9 @@
           <invertIfNegative val="0"/>
           <dLbls>
             <txPr>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr wrap="square"/>
+              <a:lstStyle/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -3823,7 +3826,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+          <a:ln w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -3832,9 +3835,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -3865,7 +3868,7 @@
         <axPos val="l"/>
         <majorGridlines>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+            <a:ln w="9360">
               <a:solidFill>
                 <a:srgbClr val="878787"/>
               </a:solidFill>
@@ -3879,7 +3882,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+          <a:ln w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -3888,9 +3891,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -3914,16 +3917,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -3943,10 +3946,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+    <a:solidFill>
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+    <a:ln w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -3958,7 +3961,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <twoCellAnchor editAs="oneCell">
     <from>
       <col>0</col>
@@ -3978,9 +3981,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+          <c:chart r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -4005,9 +4008,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+          <c:chart r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -4032,9 +4035,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
+          <c:chart r:id="rId3"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -4059,9 +4062,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
+          <c:chart r:id="rId4"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -4086,9 +4089,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId5"/>
+          <c:chart r:id="rId5"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -4113,9 +4116,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId6"/>
+          <c:chart r:id="rId6"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -4140,9 +4143,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId7"/>
+          <c:chart r:id="rId7"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -4848,6 +4851,7 @@
         <v/>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="26.25" customHeight="1" s="50">
       <c r="A4" s="89" t="inlineStr">
         <is>
@@ -6199,6 +6203,8 @@
         <v/>
       </c>
     </row>
+    <row r="17"/>
+    <row r="18"/>
     <row r="19" ht="15" customHeight="1" s="50">
       <c r="A19" s="57" t="inlineStr">
         <is>
@@ -6272,6 +6278,8 @@
         <v/>
       </c>
     </row>
+    <row r="22"/>
+    <row r="23"/>
     <row r="24" ht="15" customHeight="1" s="50">
       <c r="A24" s="57" t="inlineStr">
         <is>
@@ -6380,6 +6388,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="15" customHeight="1" s="50">
       <c r="A4" s="57" t="inlineStr">
         <is>
@@ -6403,6 +6412,7 @@
         <v/>
       </c>
     </row>
+    <row r="6"/>
     <row r="7" ht="26.25" customHeight="1" s="50">
       <c r="A7" s="60" t="inlineStr">
         <is>
@@ -6646,6 +6656,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="15" customHeight="1" s="50">
       <c r="A4" s="57" t="inlineStr">
         <is>
@@ -6704,6 +6715,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="48" customHeight="1" s="50">
       <c r="A4" s="68" t="inlineStr">
         <is>
@@ -6776,6 +6788,7 @@
         </is>
       </c>
     </row>
+    <row r="10"/>
     <row r="11" ht="15" customHeight="1" s="50">
       <c r="A11" s="57" t="inlineStr">
         <is>
@@ -6818,6 +6831,7 @@
         </is>
       </c>
     </row>
+    <row r="17"/>
     <row r="18" ht="15" customHeight="1" s="50">
       <c r="A18" s="57" t="inlineStr">
         <is>
@@ -6877,6 +6891,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="15" customHeight="1" s="50">
       <c r="A4" s="60" t="inlineStr">
         <is>
@@ -7080,6 +7095,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="15" customHeight="1" s="50">
       <c r="A3" s="60" t="inlineStr">
         <is>
@@ -7304,6 +7320,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="26.25" customHeight="1" s="50">
       <c r="A3" s="60" t="inlineStr">
         <is>
@@ -17809,7 +17826,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I164"/>
+  <dimension ref="A1:I167"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="38" customWidth="1" style="49" min="1" max="2"/>
@@ -17824,6 +17841,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="15" customHeight="1" s="50">
       <c r="A3" s="81" t="inlineStr">
         <is>
@@ -18034,6 +18052,11 @@
         <v>1</v>
       </c>
     </row>
+    <row r="10"/>
+    <row r="11"/>
+    <row r="12"/>
+    <row r="13"/>
+    <row r="14"/>
     <row r="15" ht="15" customHeight="1" s="50">
       <c r="A15" s="84" t="inlineStr">
         <is>
@@ -18041,6 +18064,7 @@
         </is>
       </c>
     </row>
+    <row r="16"/>
     <row r="17" ht="15" customHeight="1" s="50">
       <c r="A17" s="81" t="inlineStr">
         <is>
@@ -18690,6 +18714,10 @@
         </is>
       </c>
     </row>
+    <row r="36"/>
+    <row r="37"/>
+    <row r="38"/>
+    <row r="39"/>
     <row r="40" ht="15" customHeight="1" s="50">
       <c r="A40" s="77" t="n">
         <v>46196</v>
@@ -20642,123 +20670,148 @@
       </c>
     </row>
     <row r="119" ht="15" customHeight="1" s="50">
-      <c r="A119" s="84" t="inlineStr">
+      <c r="A119" s="90" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B119" s="49" t="inlineStr">
+        <is>
+          <t>Salt Shark</t>
+        </is>
+      </c>
+      <c r="C119" s="92" t="inlineStr">
+        <is>
+          <t>4938</t>
+        </is>
+      </c>
+      <c r="D119" s="92" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="E119" s="49" t="inlineStr">
+        <is>
+          <t>Order Cut Off</t>
+        </is>
+      </c>
+      <c r="F119" s="49" t="inlineStr">
+        <is>
+          <t>Count as met</t>
+        </is>
+      </c>
+      <c r="G119" s="49" t="inlineStr">
+        <is>
+          <t>Order not yet dispatched; confirmed by operations to be completed and dispatched tomorrow (2 Oct 2026) - extension approved, not a genuine cutoff miss.</t>
+        </is>
+      </c>
+    </row>
+    <row r="120" ht="15" customHeight="1" s="50">
+      <c r="A120" s="90" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B120" s="49" t="inlineStr">
+        <is>
+          <t>Salt Shark</t>
+        </is>
+      </c>
+      <c r="C120" s="92" t="inlineStr">
+        <is>
+          <t>4953</t>
+        </is>
+      </c>
+      <c r="D120" s="92" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="E120" s="49" t="inlineStr">
+        <is>
+          <t>Order Cut Off</t>
+        </is>
+      </c>
+      <c r="F120" s="49" t="inlineStr">
+        <is>
+          <t>Count as met</t>
+        </is>
+      </c>
+      <c r="G120" s="49" t="inlineStr">
+        <is>
+          <t>Order not yet dispatched; confirmed by operations to be completed and dispatched tomorrow (2 Oct 2026) - extension approved, not a genuine cutoff miss.</t>
+        </is>
+      </c>
+    </row>
+    <row r="121" ht="15" customHeight="1" s="50">
+      <c r="A121" s="90" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B121" s="49" t="inlineStr">
+        <is>
+          <t>Flo &amp; Frankie</t>
+        </is>
+      </c>
+      <c r="C121" s="92" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="D121" s="92" t="n"/>
+      <c r="E121" s="49" t="inlineStr">
+        <is>
+          <t>Order Cut Off</t>
+        </is>
+      </c>
+      <c r="F121" s="49" t="inlineStr">
+        <is>
+          <t>Count as met</t>
+        </is>
+      </c>
+      <c r="G121" s="49" t="inlineStr">
+        <is>
+          <t>Customer agreement: Flo &amp; Frankie Order Cut Off orders count as met going forward, per agreement with the customer.</t>
+        </is>
+      </c>
+    </row>
+    <row r="122" ht="15" customHeight="1" s="50">
+      <c r="A122" s="84" t="inlineStr">
         <is>
           <t>Action must be either "Exclude from calculation" or "Count as met". KPI should match the KPI name exactly (e.g. "Order Cut Off"). Order Reference must match the customer's order reference number.</t>
         </is>
       </c>
     </row>
-    <row r="120" ht="15" customHeight="1" s="50"/>
-    <row r="121">
-      <c r="A121" s="81" t="inlineStr">
+    <row r="123" ht="15" customHeight="1" s="50"/>
+    <row r="124">
+      <c r="A124" s="81" t="inlineStr">
         <is>
           <t>Order Content-Based Overrides</t>
         </is>
       </c>
     </row>
-    <row r="122">
-      <c r="A122" s="82" t="inlineStr">
+    <row r="125">
+      <c r="A125" s="82" t="inlineStr">
         <is>
           <t>Customer</t>
         </is>
-      </c>
-    </row>
-    <row r="123">
-      <c r="A123" s="49" t="inlineStr">
-        <is>
-          <t>Vixxen</t>
-        </is>
-      </c>
-      <c r="B123" s="49" t="inlineStr">
-        <is>
-          <t>Delivery Company Name</t>
-        </is>
-      </c>
-      <c r="C123" s="49" t="inlineStr">
-        <is>
-          <t>farmers</t>
-        </is>
-      </c>
-      <c r="D123" s="49" t="inlineStr">
-        <is>
-          <t>Next Tuesday (17:00)</t>
-        </is>
-      </c>
-    </row>
-    <row r="124">
-      <c r="A124" s="49" t="inlineStr">
-        <is>
-          <t>Simply Clean</t>
-        </is>
-      </c>
-      <c r="B124" s="49" t="inlineStr">
-        <is>
-          <t>Delivery Company Name</t>
-        </is>
-      </c>
-      <c r="C124" s="49" t="inlineStr">
-        <is>
-          <t>briscoes</t>
-        </is>
-      </c>
-      <c r="D124" s="49" t="inlineStr">
-        <is>
-          <t>Next Tuesday (17:00)</t>
-        </is>
-      </c>
-    </row>
-    <row r="125">
-      <c r="A125" s="49" t="inlineStr">
-        <is>
-          <t>Vixxen</t>
-        </is>
-      </c>
-      <c r="B125" s="49" t="inlineStr">
-        <is>
-          <t>Delivery Company Name</t>
-        </is>
-      </c>
-      <c r="C125" s="49" t="inlineStr">
-        <is>
-          <t>farmers</t>
-        </is>
-      </c>
-      <c r="D125" s="49" t="inlineStr">
-        <is>
-          <t>Next Monday (20:00)</t>
-        </is>
-      </c>
-      <c r="E125" s="83" t="n">
-        <v>46251</v>
-      </c>
-      <c r="F125" s="83" t="n">
-        <v>46254</v>
       </c>
     </row>
     <row r="126" ht="126.85" customHeight="1" s="50">
       <c r="A126" s="49" t="inlineStr">
         <is>
-          <t>Gym Equip</t>
+          <t>Vixxen</t>
         </is>
       </c>
       <c r="B126" s="49" t="inlineStr">
         <is>
-          <t>All Orders</t>
+          <t>Delivery Company Name</t>
         </is>
       </c>
       <c r="C126" s="49" t="inlineStr">
         <is>
-          <t>all</t>
+          <t>farmers</t>
         </is>
       </c>
       <c r="D126" s="49" t="inlineStr">
         <is>
-          <t>Fixed (2026-09-02 20:00)</t>
-        </is>
-      </c>
-      <c r="E126" s="83" t="n"/>
-      <c r="F126" s="83" t="n">
-        <v>46266</v>
+          <t>Next Tuesday (17:00)</t>
+        </is>
       </c>
     </row>
     <row r="127">
@@ -20774,115 +20827,159 @@
       </c>
       <c r="C127" s="49" t="inlineStr">
         <is>
+          <t>briscoes</t>
+        </is>
+      </c>
+      <c r="D127" s="49" t="inlineStr">
+        <is>
+          <t>Next Tuesday (17:00)</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="49" t="inlineStr">
+        <is>
+          <t>Vixxen</t>
+        </is>
+      </c>
+      <c r="B128" s="49" t="inlineStr">
+        <is>
+          <t>Delivery Company Name</t>
+        </is>
+      </c>
+      <c r="C128" s="49" t="inlineStr">
+        <is>
+          <t>farmers</t>
+        </is>
+      </c>
+      <c r="D128" s="49" t="inlineStr">
+        <is>
+          <t>Next Monday (20:00)</t>
+        </is>
+      </c>
+      <c r="E128" s="83" t="n">
+        <v>46251</v>
+      </c>
+      <c r="F128" s="83" t="n">
+        <v>46254</v>
+      </c>
+    </row>
+    <row r="129" ht="126.85" customHeight="1" s="50">
+      <c r="A129" s="49" t="inlineStr">
+        <is>
+          <t>Gym Equip</t>
+        </is>
+      </c>
+      <c r="B129" s="49" t="inlineStr">
+        <is>
+          <t>All Orders</t>
+        </is>
+      </c>
+      <c r="C129" s="49" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="D129" s="49" t="inlineStr">
+        <is>
+          <t>Fixed (2026-09-02 20:00)</t>
+        </is>
+      </c>
+      <c r="E129" s="83" t="n"/>
+      <c r="F129" s="83" t="n">
+        <v>46266</v>
+      </c>
+    </row>
+    <row r="130" ht="15" customHeight="1" s="50">
+      <c r="A130" s="49" t="inlineStr">
+        <is>
+          <t>Simply Clean</t>
+        </is>
+      </c>
+      <c r="B130" s="49" t="inlineStr">
+        <is>
+          <t>Delivery Company Name</t>
+        </is>
+      </c>
+      <c r="C130" s="49" t="inlineStr">
+        <is>
           <t>briscoes group</t>
         </is>
       </c>
-      <c r="D127" s="49" t="inlineStr">
+      <c r="D130" s="49" t="inlineStr">
         <is>
           <t>Fixed (2026-09-18 20:00)</t>
         </is>
       </c>
-      <c r="E127" s="83" t="n">
+      <c r="E130" s="83" t="n">
         <v>46280</v>
       </c>
-      <c r="F127" s="83" t="n">
+      <c r="F130" s="83" t="n">
         <v>46280</v>
       </c>
     </row>
-    <row r="129" ht="15" customHeight="1" s="50"/>
-    <row r="130" ht="15" customHeight="1" s="50"/>
-    <row r="131" ht="23.85" customHeight="1" s="50"/>
+    <row r="131" ht="23.85" customHeight="1" s="50">
+      <c r="A131" s="49" t="inlineStr">
+        <is>
+          <t>Vixxen</t>
+        </is>
+      </c>
+      <c r="B131" s="49" t="inlineStr">
+        <is>
+          <t>Delivery Company Name</t>
+        </is>
+      </c>
+      <c r="C131" s="49" t="inlineStr">
+        <is>
+          <t>farmers</t>
+        </is>
+      </c>
+      <c r="D131" s="49" t="inlineStr">
+        <is>
+          <t>Fixed (2026-10-13 20:00)</t>
+        </is>
+      </c>
+      <c r="E131" s="83" t="n">
+        <v>46300</v>
+      </c>
+      <c r="F131" s="83" t="n">
+        <v>46300</v>
+      </c>
+    </row>
     <row r="132" ht="15" customHeight="1" s="50"/>
-    <row r="133" ht="23.85" customHeight="1" s="50">
-      <c r="A133" s="84" t="inlineStr">
+    <row r="133" ht="15" customHeight="1" s="50"/>
+    <row r="134" ht="23.85" customHeight="1" s="50"/>
+    <row r="135" ht="15" customHeight="1" s="50"/>
+    <row r="136" ht="23.85" customHeight="1" s="50">
+      <c r="A136" s="84" t="inlineStr">
         <is>
           <t>Match Field currently supports "Delivery Company Name" or "All Orders" (matches every order for that customer, regardless of content - use with Contains="all"). Deadline Rule may be "Same day", "Next business day (EOD)", "Next &lt;Weekday&gt; (&lt;time&gt;)" e.g. "Next Tuesday (5pm)" - the next occurrence of that weekday on/after the order's creation date, at the given NZ time - or "Fixed (&lt;YYYY-MM-DD HH:MM&gt;)" for a single absolute deadline applied to every order in the effective window (e.g. a customer-wide stock hold/customs embargo). Leave Effective From/To blank to apply to all dates.</t>
         </is>
       </c>
     </row>
-    <row r="134" ht="23.85" customHeight="1" s="50"/>
-    <row r="136" ht="99.95" customHeight="1" s="50">
-      <c r="A136" s="85" t="inlineStr">
+    <row r="137" ht="23.85" customHeight="1" s="50"/>
+    <row r="138"/>
+    <row r="139" ht="99.95" customHeight="1" s="50">
+      <c r="A139" s="85" t="inlineStr">
         <is>
           <t>Table 4: DIFOT Delivery Recipient Exceptions</t>
         </is>
       </c>
     </row>
-    <row r="137">
-      <c r="A137" s="86" t="inlineStr">
+    <row r="140" ht="15" customHeight="1" s="50">
+      <c r="A140" s="86" t="inlineStr">
         <is>
           <t>Match Field</t>
         </is>
       </c>
-      <c r="F137" s="86" t="inlineStr">
+      <c r="F140" s="86" t="inlineStr">
         <is>
           <t>Attribute To</t>
         </is>
       </c>
-      <c r="G137" s="86" t="inlineStr">
+      <c r="G140" s="86" t="inlineStr">
         <is>
           <t>Reason</t>
-        </is>
-      </c>
-    </row>
-    <row r="138">
-      <c r="A138" s="49" t="inlineStr">
-        <is>
-          <t>ShipTo</t>
-        </is>
-      </c>
-      <c r="B138" s="49" t="inlineStr">
-        <is>
-          <t>supercheap</t>
-        </is>
-      </c>
-      <c r="C138" s="49" t="inlineStr">
-        <is>
-          <t>Count as met</t>
-        </is>
-      </c>
-      <c r="F138" s="49" t="inlineStr">
-        <is>
-          <t>Oricom</t>
-        </is>
-      </c>
-      <c r="G138" s="69" t="inlineStr">
-        <is>
-          <t>Supercheap Auto/Retail DC orders use separate pre-arranged bookings, not standard carrier tracking</t>
-        </is>
-      </c>
-    </row>
-    <row r="139" ht="15" customHeight="1" s="50">
-      <c r="A139" s="49" t="inlineStr">
-        <is>
-          <t>ShipTo</t>
-        </is>
-      </c>
-    </row>
-    <row r="140" ht="15" customHeight="1" s="50">
-      <c r="A140" s="49" t="inlineStr">
-        <is>
-          <t>ShipTo</t>
-        </is>
-      </c>
-      <c r="B140" s="49" t="inlineStr">
-        <is>
-          <t>srg</t>
-        </is>
-      </c>
-      <c r="C140" s="49" t="inlineStr">
-        <is>
-          <t>Count as met</t>
-        </is>
-      </c>
-      <c r="F140" s="49" t="inlineStr">
-        <is>
-          <t>Oricom</t>
-        </is>
-      </c>
-      <c r="G140" s="69" t="inlineStr">
-        <is>
-          <t>SRG (Super Retail Group) DC orders use separate pre-arranged bookings</t>
         </is>
       </c>
     </row>
@@ -20894,171 +20991,238 @@
       </c>
       <c r="B141" s="49" t="inlineStr">
         <is>
+          <t>supercheap</t>
+        </is>
+      </c>
+      <c r="C141" s="49" t="inlineStr">
+        <is>
+          <t>Count as met</t>
+        </is>
+      </c>
+      <c r="F141" s="49" t="inlineStr">
+        <is>
+          <t>Oricom</t>
+        </is>
+      </c>
+      <c r="G141" s="69" t="inlineStr">
+        <is>
+          <t>Supercheap Auto/Retail DC orders use separate pre-arranged bookings, not standard carrier tracking</t>
+        </is>
+      </c>
+    </row>
+    <row r="142" ht="15" customHeight="1" s="50">
+      <c r="A142" s="49" t="inlineStr">
+        <is>
+          <t>ShipTo</t>
+        </is>
+      </c>
+    </row>
+    <row r="143" ht="15" customHeight="1" s="50">
+      <c r="A143" s="49" t="inlineStr">
+        <is>
+          <t>ShipTo</t>
+        </is>
+      </c>
+      <c r="B143" s="49" t="inlineStr">
+        <is>
+          <t>srg</t>
+        </is>
+      </c>
+      <c r="C143" s="49" t="inlineStr">
+        <is>
+          <t>Count as met</t>
+        </is>
+      </c>
+      <c r="F143" s="49" t="inlineStr">
+        <is>
+          <t>Oricom</t>
+        </is>
+      </c>
+      <c r="G143" s="69" t="inlineStr">
+        <is>
+          <t>SRG (Super Retail Group) DC orders use separate pre-arranged bookings</t>
+        </is>
+      </c>
+    </row>
+    <row r="144" ht="68.65000000000001" customHeight="1" s="50">
+      <c r="A144" s="49" t="inlineStr">
+        <is>
+          <t>ShipTo</t>
+        </is>
+      </c>
+      <c r="B144" s="49" t="inlineStr">
+        <is>
           <t>repco</t>
         </is>
       </c>
-      <c r="C141" s="49" t="inlineStr">
+      <c r="C144" s="49" t="inlineStr">
         <is>
           <t>Count as met</t>
         </is>
       </c>
-      <c r="F141" s="49" t="inlineStr">
+      <c r="F144" s="49" t="inlineStr">
         <is>
           <t>Oricom</t>
         </is>
       </c>
-      <c r="G141" s="69" t="inlineStr">
+      <c r="G144" s="69" t="inlineStr">
         <is>
           <t>Repco (GPC-owned) orders use separate pre-arranged bookings</t>
         </is>
       </c>
     </row>
-    <row r="143" ht="46.25" customHeight="1" s="50">
-      <c r="A143" s="87" t="inlineStr">
+    <row r="145"/>
+    <row r="146" ht="46.25" customHeight="1" s="50">
+      <c r="A146" s="87" t="inlineStr">
         <is>
           <t>Match Field "ShipTo" checks the Starshipit ShipTo field (case-insensitive substring match). Action "Count as met" includes these orders in the DIFOT denominator and marks them as on-time, regardless of tracking status or actual delivery date. "Attribute To" sets the customer these orders are attributed to directly (bypassing the CartonCloud join), which is needed for pre-integration DC orders where the Starshipit TheirRef does not correspond to a CC numericId. Action "Exclude" removes the order from the DIFOT calculation entirely.</t>
         </is>
       </c>
     </row>
-    <row r="146" ht="15" customHeight="1" s="50">
-      <c r="A146" s="85" t="inlineStr">
+    <row r="147" ht="15" customHeight="1" s="50"/>
+    <row r="148" ht="15" customHeight="1" s="50"/>
+    <row r="149" ht="15" customHeight="1" s="50">
+      <c r="A149" s="85" t="inlineStr">
         <is>
           <t>Table 5: International Carrier SLAs</t>
         </is>
       </c>
     </row>
-    <row r="147" ht="15" customHeight="1" s="50">
-      <c r="A147" s="86" t="inlineStr">
+    <row r="150" ht="15" customHeight="1" s="50">
+      <c r="A150" s="86" t="inlineStr">
         <is>
           <t>Service Code</t>
         </is>
       </c>
-      <c r="B147" s="86" t="inlineStr">
+      <c r="B150" s="86" t="inlineStr">
         <is>
           <t>Destination</t>
         </is>
       </c>
-      <c r="C147" s="86" t="inlineStr">
+      <c r="C150" s="86" t="inlineStr">
         <is>
           <t>Business Days</t>
         </is>
       </c>
-      <c r="D147" s="86" t="inlineStr">
+      <c r="D150" s="86" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
       </c>
-      <c r="E147" s="86" t="inlineStr">
+      <c r="E150" s="86" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
-    <row r="148" ht="15" customHeight="1" s="50">
-      <c r="A148" s="49" t="inlineStr">
+    <row r="151" ht="15" customHeight="1" s="50">
+      <c r="A151" s="49" t="inlineStr">
         <is>
           <t>FEDEX_INTERNATIONAL_CONNECT_PLUS</t>
         </is>
       </c>
-      <c r="B148" s="49" t="inlineStr">
+      <c r="B151" s="49" t="inlineStr">
         <is>
           <t>All international</t>
         </is>
       </c>
-      <c r="C148" s="49" t="n">
+      <c r="C151" s="49" t="n">
         <v>3</v>
       </c>
-      <c r="D148" s="49" t="inlineStr">
+      <c r="D151" s="49" t="inlineStr">
         <is>
           <t>fedex.com/en-nz</t>
         </is>
       </c>
-      <c r="E148" s="69" t="inlineStr">
+      <c r="E151" s="69" t="inlineStr">
         <is>
           <t>FedEx FICP 'typically 2-3 business days worldwide' - using maximum per FP policy</t>
         </is>
       </c>
     </row>
-    <row r="149" ht="15" customHeight="1" s="50"/>
-    <row r="150">
-      <c r="A150" s="87" t="inlineStr">
+    <row r="152" ht="15" customHeight="1" s="50"/>
+    <row r="153" ht="15" customHeight="1" s="50">
+      <c r="A153" s="87" t="inlineStr">
         <is>
           <t>Business Days are calculated from pickup date using add_business_days() (Mon-Fri only). To add a new carrier/destination rule, add a row here and update extract_difot.py INTL_CARRIER_DAYS dict. If a range is published (e.g. 3-5 days), always use the maximum.</t>
         </is>
       </c>
     </row>
-    <row r="151" ht="15" customHeight="1" s="50"/>
-    <row r="153" ht="15" customHeight="1" s="50">
-      <c r="A153" s="49" t="inlineStr">
+    <row r="154" ht="15" customHeight="1" s="50"/>
+    <row r="155" ht="15" customHeight="1" s="50"/>
+    <row r="156" ht="15" customHeight="1" s="50">
+      <c r="A156" s="49" t="inlineStr">
         <is>
           <t>Table 6: Public Holidays</t>
         </is>
       </c>
     </row>
-    <row r="154" ht="15" customHeight="1" s="50">
-      <c r="A154" s="49" t="inlineStr">
+    <row r="157" ht="15" customHeight="1" s="50">
+      <c r="A157" s="49" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="B154" s="49" t="inlineStr">
+      <c r="B157" s="49" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
-    <row r="155" ht="15" customHeight="1" s="50">
-      <c r="A155" s="77" t="n">
+    <row r="158" ht="15" customHeight="1" s="50">
+      <c r="A158" s="77" t="n">
         <v>46213</v>
       </c>
-      <c r="B155" s="49" t="inlineStr">
+      <c r="B158" s="49" t="inlineStr">
         <is>
           <t>Wellington Anniversary / regional public holiday — deadlines falling on this day roll to next business day</t>
         </is>
       </c>
     </row>
-    <row r="156">
-      <c r="A156" s="83" t="n"/>
-    </row>
-    <row r="157" ht="15" customHeight="1" s="50"/>
-    <row r="158">
-      <c r="A158" s="49" t="inlineStr">
-        <is>
-          <t>Add future public holidays here. Deadlines (Order Cut Off, required delivery date) that fall on a listed date will automatically roll forward to the next business day.</t>
-        </is>
-      </c>
-    </row>
-    <row r="160">
-      <c r="A160" s="49" t="inlineStr">
-        <is>
-          <t>Table 7: Operational Exceptions (Non-Business Days)</t>
-        </is>
-      </c>
-    </row>
+    <row r="159">
+      <c r="A159" s="83" t="n"/>
+    </row>
+    <row r="160" ht="15" customHeight="1" s="50"/>
     <row r="161">
       <c r="A161" s="49" t="inlineStr">
         <is>
-          <t>Date</t>
-        </is>
-      </c>
-      <c r="B161" s="49" t="inlineStr">
-        <is>
-          <t>Reason</t>
-        </is>
-      </c>
-    </row>
-    <row r="162">
-      <c r="A162" s="83" t="n">
-        <v>46244</v>
-      </c>
-      <c r="B162" s="49" t="inlineStr">
-        <is>
-          <t>Warehouse fibre/network outage - unable to process orders all day. NOT a public holiday - an operational disruption logged here so KPI deadline calculations treat it the same way a public holiday is treated (Order Cut Off and required-delivery-date deadlines roll to the next genuine business day; no orders penalised for lack of processing today).</t>
+          <t>Add future public holidays here. Deadlines (Order Cut Off, required delivery date) that fall on a listed date will automatically roll forward to the next business day.</t>
+        </is>
+      </c>
+    </row>
+    <row r="162"/>
+    <row r="163">
+      <c r="A163" s="49" t="inlineStr">
+        <is>
+          <t>Table 7: Operational Exceptions (Non-Business Days)</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" s="49" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B164" s="49" t="inlineStr">
+        <is>
+          <t>Reason</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" s="83" t="n">
+        <v>46244</v>
+      </c>
+      <c r="B165" s="49" t="inlineStr">
+        <is>
+          <t>Warehouse fibre/network outage - unable to process orders all day. NOT a public holiday - an operational disruption logged here so KPI deadline calculations treat it the same way a public holiday is treated (Order Cut Off and required-delivery-date deadlines roll to the next genuine business day; no orders penalised for lack of processing today).</t>
+        </is>
+      </c>
+    </row>
+    <row r="166"/>
+    <row r="167">
+      <c r="A167" s="49" t="inlineStr">
         <is>
           <t>Add one-off operational disruptions here (e.g. system outages, warehouse closures) that should count as a non-business day for KPI deadlines without being recorded as an actual public holiday. Functions identically to Table 6 for deadline-rolling purposes.</t>
         </is>
@@ -21109,6 +21273,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="15" customHeight="1" s="50">
       <c r="A4" s="82" t="inlineStr">
         <is>
@@ -21301,20 +21466,20 @@
       <c r="A12" s="91" t="n">
         <v>46295</v>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B12" s="49" t="inlineStr">
         <is>
           <t>Vixxen</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C12" s="49" t="inlineStr">
         <is>
           <t>3380</t>
         </is>
       </c>
-      <c r="D12" t="n">
+      <c r="D12" s="49" t="n">
         <v>7</v>
       </c>
-      <c r="E12" t="inlineStr">
+      <c r="E12" s="49" t="inlineStr">
         <is>
           <t>Cross-labelled shipping labels - items picked accurately but shipped to wrong destination due to label mix-up</t>
         </is>
@@ -21324,20 +21489,20 @@
       <c r="A13" s="91" t="n">
         <v>46295</v>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B13" s="49" t="inlineStr">
         <is>
           <t>Vixxen</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="C13" s="49" t="inlineStr">
         <is>
           <t>3378</t>
         </is>
       </c>
-      <c r="D13" t="n">
+      <c r="D13" s="49" t="n">
         <v>7</v>
       </c>
-      <c r="E13" t="inlineStr">
+      <c r="E13" s="49" t="inlineStr">
         <is>
           <t>Cross-labelled shipping labels - items picked accurately but shipped to wrong destination due to label mix-up</t>
         </is>
@@ -21351,255 +21516,4 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
 </worksheet>
-</file>
-
-<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100CB702797C59B384BA5825BD7F91C8FA6" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ed5aae9864b7dcbba9993313f29ed662">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="7e670929-1bdc-480c-8510-e43a2a862a6e" xmlns:ns3="e1750f8f-64a8-40e8-9e0c-21710cc1a7bb" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="59a292da2c54c23b9d44e0544df2ef32" ns2:_="" ns3:_="">
-    <xsd:import namespace="7e670929-1bdc-480c-8510-e43a2a862a6e"/>
-    <xsd:import namespace="e1750f8f-64a8-40e8-9e0c-21710cc1a7bb"/>
-    <xsd:element name="properties">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element name="documentManagement">
-            <xsd:complexType>
-              <xsd:all>
-                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
-                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
-                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
-                <xsd:element ref="ns2:Access" minOccurs="0"/>
-                <xsd:element ref="ns2:Access_x002f_Info" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceLocation" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
-              </xsd:all>
-            </xsd:complexType>
-          </xsd:element>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="7e670929-1bdc-480c-8510-e43a2a862a6e" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceSearchProperties" ma:index="10" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceDateTaken" ma:index="11" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="13" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="b25c28e6-01a0-48d2-b828-62504f505dd7" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="MediaServiceOCR" ma:index="15" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceGenerationTime" ma:index="16" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceEventHashCode" ma:index="17" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="Access" ma:index="18" nillable="true" ma:displayName="Access" ma:description="Who gets access&#10;" ma:format="Dropdown" ma:internalName="Access">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="Access_x002f_Info" ma:index="19" nillable="true" ma:displayName="Access/ Info " ma:format="Dropdown" ma:internalName="Access_x002f_Info">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceLocation" ma:index="20" nillable="true" ma:displayName="Location" ma:indexed="true" ma:internalName="MediaServiceLocation" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaLengthInSeconds" ma:index="21" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Unknown"/>
-      </xsd:simpleType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="e1750f8f-64a8-40e8-9e0c-21710cc1a7bb" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="TaxCatchAll" ma:index="14" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{156fa16d-c7d6-4694-aac4-2bac9e86d8b0}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="e1750f8f-64a8-40e8-9e0c-21710cc1a7bb">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:MultiChoiceLookup">
-            <xsd:sequence>
-              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
-    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
-    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
-    <xsd:element name="coreProperties" type="CT_coreProperties"/>
-    <xsd:complexType name="CT_coreProperties">
-      <xsd:all>
-        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
-        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
-        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
-          <xsd:annotation>
-            <xsd:documentation>
-                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
-                    </xsd:documentation>
-          </xsd:annotation>
-        </xsd:element>
-        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-      </xsd:all>
-    </xsd:complexType>
-  </xsd:schema>
-  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
-    <xs:element name="Person">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:DisplayName" minOccurs="0"/>
-          <xs:element ref="pc:AccountId" minOccurs="0"/>
-          <xs:element ref="pc:AccountType" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="DisplayName" type="xs:string"/>
-    <xs:element name="AccountId" type="xs:string"/>
-    <xs:element name="AccountType" type="xs:string"/>
-    <xs:element name="BDCAssociatedEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-        <xs:attribute ref="pc:EntityNamespace"/>
-        <xs:attribute ref="pc:EntityName"/>
-        <xs:attribute ref="pc:SystemInstanceName"/>
-        <xs:attribute ref="pc:AssociationName"/>
-      </xs:complexType>
-    </xs:element>
-    <xs:attribute name="EntityNamespace" type="xs:string"/>
-    <xs:attribute name="EntityName" type="xs:string"/>
-    <xs:attribute name="SystemInstanceName" type="xs:string"/>
-    <xs:attribute name="AssociationName" type="xs:string"/>
-    <xs:element name="BDCEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
-          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
-          <xs:element ref="pc:EntityId1" minOccurs="0"/>
-          <xs:element ref="pc:EntityId2" minOccurs="0"/>
-          <xs:element ref="pc:EntityId3" minOccurs="0"/>
-          <xs:element ref="pc:EntityId4" minOccurs="0"/>
-          <xs:element ref="pc:EntityId5" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="EntityDisplayName" type="xs:string"/>
-    <xs:element name="EntityInstanceReference" type="xs:string"/>
-    <xs:element name="EntityId1" type="xs:string"/>
-    <xs:element name="EntityId2" type="xs:string"/>
-    <xs:element name="EntityId3" type="xs:string"/>
-    <xs:element name="EntityId4" type="xs:string"/>
-    <xs:element name="EntityId5" type="xs:string"/>
-    <xs:element name="Terms">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermInfo">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermName" minOccurs="0"/>
-          <xs:element ref="pc:TermId" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermName" type="xs:string"/>
-    <xs:element name="TermId" type="xs:string"/>
-  </xs:schema>
-</ct:contentTypeSchema>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <Access xmlns="7e670929-1bdc-480c-8510-e43a2a862a6e" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="7e670929-1bdc-480c-8510-e43a2a862a6e">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="e1750f8f-64a8-40e8-9e0c-21710cc1a7bb" xsi:nil="true"/>
-    <Access_x002f_Info xmlns="7e670929-1bdc-480c-8510-e43a2a862a6e" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{945D8665-BB08-45C8-840D-18D1435796C1}"/>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4BD9ABE0-6CF6-4F1E-898D-882E0269A924}"/>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{03B5FEB4-9DED-4683-B971-45C8DEFC8855}"/>
 </file>
</xml_diff>

<commit_message>
Log Coromandel Mountains cross-labelled cartons 5311 and 5312 (#2)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Co-authored-by: Mike-FulfilmentPlus <330614259+Mike-FulfilmentPlus@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/pipeline/kpi_dashboard.xlsx
+++ b/pipeline/kpi_dashboard.xlsx
@@ -17266,30 +17266,30 @@
       <c r="A353" s="90" t="n">
         <v>46266</v>
       </c>
-      <c r="B353" t="inlineStr">
+      <c r="B353" s="49" t="inlineStr">
         <is>
           <t>Aleger Studio</t>
         </is>
       </c>
-      <c r="C353" t="inlineStr">
+      <c r="C353" s="49" t="inlineStr">
         <is>
           <t>Freight DIFOT</t>
         </is>
       </c>
-      <c r="E353" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="F353" t="n">
+      <c r="E353" s="49" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="F353" s="49" t="n">
         <v>6</v>
       </c>
-      <c r="G353" t="n">
+      <c r="G353" s="49" t="n">
         <v>6</v>
       </c>
-      <c r="H353">
+      <c r="H353" s="49">
         <f>F353/G353</f>
         <v/>
       </c>
-      <c r="I353">
+      <c r="I353" s="49">
         <f>IF(H353&gt;=E353,"Yes","No")</f>
         <v/>
       </c>
@@ -17298,34 +17298,34 @@
       <c r="A354" s="90" t="n">
         <v>46266</v>
       </c>
-      <c r="B354" t="inlineStr">
+      <c r="B354" s="49" t="inlineStr">
         <is>
           <t>Coromandel Mountains Company Limited</t>
         </is>
       </c>
-      <c r="C354" t="inlineStr">
+      <c r="C354" s="49" t="inlineStr">
         <is>
           <t>Freight DIFOT</t>
         </is>
       </c>
-      <c r="E354" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="F354" t="n">
+      <c r="E354" s="49" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="F354" s="49" t="n">
         <v>36</v>
       </c>
-      <c r="G354" t="n">
+      <c r="G354" s="49" t="n">
         <v>38</v>
       </c>
-      <c r="H354">
+      <c r="H354" s="49">
         <f>F354/G354</f>
         <v/>
       </c>
-      <c r="I354">
+      <c r="I354" s="49">
         <f>IF(H354&gt;=E354,"Yes","No")</f>
         <v/>
       </c>
-      <c r="J354" t="inlineStr">
+      <c r="J354" s="49" t="inlineStr">
         <is>
           <t>Below target - investigate root cause and add to next month's action plan</t>
         </is>
@@ -17335,34 +17335,34 @@
       <c r="A355" s="90" t="n">
         <v>46266</v>
       </c>
-      <c r="B355" t="inlineStr">
+      <c r="B355" s="49" t="inlineStr">
         <is>
           <t>EcoPallets</t>
         </is>
       </c>
-      <c r="C355" t="inlineStr">
+      <c r="C355" s="49" t="inlineStr">
         <is>
           <t>Freight DIFOT</t>
         </is>
       </c>
-      <c r="E355" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="F355" t="n">
+      <c r="E355" s="49" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="F355" s="49" t="n">
         <v>6</v>
       </c>
-      <c r="G355" t="n">
+      <c r="G355" s="49" t="n">
         <v>7</v>
       </c>
-      <c r="H355">
+      <c r="H355" s="49">
         <f>F355/G355</f>
         <v/>
       </c>
-      <c r="I355">
+      <c r="I355" s="49">
         <f>IF(H355&gt;=E355,"Yes","No")</f>
         <v/>
       </c>
-      <c r="J355" t="inlineStr">
+      <c r="J355" s="49" t="inlineStr">
         <is>
           <t>Below target - investigate root cause and add to next month's action plan</t>
         </is>
@@ -17372,34 +17372,34 @@
       <c r="A356" s="90" t="n">
         <v>46266</v>
       </c>
-      <c r="B356" t="inlineStr">
+      <c r="B356" s="49" t="inlineStr">
         <is>
           <t>Flo &amp; Frankie</t>
         </is>
       </c>
-      <c r="C356" t="inlineStr">
+      <c r="C356" s="49" t="inlineStr">
         <is>
           <t>Freight DIFOT</t>
         </is>
       </c>
-      <c r="E356" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="F356" t="n">
+      <c r="E356" s="49" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="F356" s="49" t="n">
         <v>11</v>
       </c>
-      <c r="G356" t="n">
+      <c r="G356" s="49" t="n">
         <v>13</v>
       </c>
-      <c r="H356">
+      <c r="H356" s="49">
         <f>F356/G356</f>
         <v/>
       </c>
-      <c r="I356">
+      <c r="I356" s="49">
         <f>IF(H356&gt;=E356,"Yes","No")</f>
         <v/>
       </c>
-      <c r="J356" t="inlineStr">
+      <c r="J356" s="49" t="inlineStr">
         <is>
           <t>Below target - investigate root cause and add to next month's action plan</t>
         </is>
@@ -17409,34 +17409,34 @@
       <c r="A357" s="90" t="n">
         <v>46266</v>
       </c>
-      <c r="B357" t="inlineStr">
+      <c r="B357" s="49" t="inlineStr">
         <is>
           <t>Gym Equip</t>
         </is>
       </c>
-      <c r="C357" t="inlineStr">
+      <c r="C357" s="49" t="inlineStr">
         <is>
           <t>Freight DIFOT</t>
         </is>
       </c>
-      <c r="E357" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="F357" t="n">
+      <c r="E357" s="49" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="F357" s="49" t="n">
         <v>17</v>
       </c>
-      <c r="G357" t="n">
+      <c r="G357" s="49" t="n">
         <v>19</v>
       </c>
-      <c r="H357">
+      <c r="H357" s="49">
         <f>F357/G357</f>
         <v/>
       </c>
-      <c r="I357">
+      <c r="I357" s="49">
         <f>IF(H357&gt;=E357,"Yes","No")</f>
         <v/>
       </c>
-      <c r="J357" t="inlineStr">
+      <c r="J357" s="49" t="inlineStr">
         <is>
           <t>Below target - investigate root cause and add to next month's action plan</t>
         </is>
@@ -17446,30 +17446,30 @@
       <c r="A358" s="90" t="n">
         <v>46266</v>
       </c>
-      <c r="B358" t="inlineStr">
+      <c r="B358" s="49" t="inlineStr">
         <is>
           <t>Interior Images</t>
         </is>
       </c>
-      <c r="C358" t="inlineStr">
+      <c r="C358" s="49" t="inlineStr">
         <is>
           <t>Freight DIFOT</t>
         </is>
       </c>
-      <c r="E358" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="F358" t="n">
+      <c r="E358" s="49" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="F358" s="49" t="n">
         <v>1</v>
       </c>
-      <c r="G358" t="n">
+      <c r="G358" s="49" t="n">
         <v>1</v>
       </c>
-      <c r="H358">
+      <c r="H358" s="49">
         <f>F358/G358</f>
         <v/>
       </c>
-      <c r="I358">
+      <c r="I358" s="49">
         <f>IF(H358&gt;=E358,"Yes","No")</f>
         <v/>
       </c>
@@ -17478,34 +17478,34 @@
       <c r="A359" s="90" t="n">
         <v>46266</v>
       </c>
-      <c r="B359" t="inlineStr">
+      <c r="B359" s="49" t="inlineStr">
         <is>
           <t>Jock Freight - SECA</t>
         </is>
       </c>
-      <c r="C359" t="inlineStr">
+      <c r="C359" s="49" t="inlineStr">
         <is>
           <t>Freight DIFOT</t>
         </is>
       </c>
-      <c r="E359" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="F359" t="n">
+      <c r="E359" s="49" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="F359" s="49" t="n">
         <v>8</v>
       </c>
-      <c r="G359" t="n">
+      <c r="G359" s="49" t="n">
         <v>9</v>
       </c>
-      <c r="H359">
+      <c r="H359" s="49">
         <f>F359/G359</f>
         <v/>
       </c>
-      <c r="I359">
+      <c r="I359" s="49">
         <f>IF(H359&gt;=E359,"Yes","No")</f>
         <v/>
       </c>
-      <c r="J359" t="inlineStr">
+      <c r="J359" s="49" t="inlineStr">
         <is>
           <t>Below target - investigate root cause and add to next month's action plan</t>
         </is>
@@ -17515,30 +17515,30 @@
       <c r="A360" s="90" t="n">
         <v>46266</v>
       </c>
-      <c r="B360" t="inlineStr">
+      <c r="B360" s="49" t="inlineStr">
         <is>
           <t>Logwin - Sikla</t>
         </is>
       </c>
-      <c r="C360" t="inlineStr">
+      <c r="C360" s="49" t="inlineStr">
         <is>
           <t>Freight DIFOT</t>
         </is>
       </c>
-      <c r="E360" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="F360" t="n">
+      <c r="E360" s="49" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="F360" s="49" t="n">
         <v>6</v>
       </c>
-      <c r="G360" t="n">
+      <c r="G360" s="49" t="n">
         <v>6</v>
       </c>
-      <c r="H360">
+      <c r="H360" s="49">
         <f>F360/G360</f>
         <v/>
       </c>
-      <c r="I360">
+      <c r="I360" s="49">
         <f>IF(H360&gt;=E360,"Yes","No")</f>
         <v/>
       </c>
@@ -17547,30 +17547,30 @@
       <c r="A361" s="90" t="n">
         <v>46266</v>
       </c>
-      <c r="B361" t="inlineStr">
+      <c r="B361" s="49" t="inlineStr">
         <is>
           <t>Made Group NZ</t>
         </is>
       </c>
-      <c r="C361" t="inlineStr">
+      <c r="C361" s="49" t="inlineStr">
         <is>
           <t>Freight DIFOT</t>
         </is>
       </c>
-      <c r="E361" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="F361" t="n">
+      <c r="E361" s="49" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="F361" s="49" t="n">
         <v>4</v>
       </c>
-      <c r="G361" t="n">
+      <c r="G361" s="49" t="n">
         <v>4</v>
       </c>
-      <c r="H361">
+      <c r="H361" s="49">
         <f>F361/G361</f>
         <v/>
       </c>
-      <c r="I361">
+      <c r="I361" s="49">
         <f>IF(H361&gt;=E361,"Yes","No")</f>
         <v/>
       </c>
@@ -17579,30 +17579,30 @@
       <c r="A362" s="90" t="n">
         <v>46266</v>
       </c>
-      <c r="B362" t="inlineStr">
+      <c r="B362" s="49" t="inlineStr">
         <is>
           <t>May Eleven NZ</t>
         </is>
       </c>
-      <c r="C362" t="inlineStr">
+      <c r="C362" s="49" t="inlineStr">
         <is>
           <t>Freight DIFOT</t>
         </is>
       </c>
-      <c r="E362" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="F362" t="n">
+      <c r="E362" s="49" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="F362" s="49" t="n">
         <v>2</v>
       </c>
-      <c r="G362" t="n">
+      <c r="G362" s="49" t="n">
         <v>2</v>
       </c>
-      <c r="H362">
+      <c r="H362" s="49">
         <f>F362/G362</f>
         <v/>
       </c>
-      <c r="I362">
+      <c r="I362" s="49">
         <f>IF(H362&gt;=E362,"Yes","No")</f>
         <v/>
       </c>
@@ -17611,34 +17611,34 @@
       <c r="A363" s="90" t="n">
         <v>46266</v>
       </c>
-      <c r="B363" t="inlineStr">
+      <c r="B363" s="49" t="inlineStr">
         <is>
           <t>Oricom</t>
         </is>
       </c>
-      <c r="C363" t="inlineStr">
+      <c r="C363" s="49" t="inlineStr">
         <is>
           <t>Freight DIFOT</t>
         </is>
       </c>
-      <c r="E363" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="F363" t="n">
+      <c r="E363" s="49" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="F363" s="49" t="n">
         <v>84</v>
       </c>
-      <c r="G363" t="n">
+      <c r="G363" s="49" t="n">
         <v>91</v>
       </c>
-      <c r="H363">
+      <c r="H363" s="49">
         <f>F363/G363</f>
         <v/>
       </c>
-      <c r="I363">
+      <c r="I363" s="49">
         <f>IF(H363&gt;=E363,"Yes","No")</f>
         <v/>
       </c>
-      <c r="J363" t="inlineStr">
+      <c r="J363" s="49" t="inlineStr">
         <is>
           <t>Below target - investigate root cause and add to next month's action plan</t>
         </is>
@@ -17648,34 +17648,34 @@
       <c r="A364" s="90" t="n">
         <v>46266</v>
       </c>
-      <c r="B364" t="inlineStr">
+      <c r="B364" s="49" t="inlineStr">
         <is>
           <t>Purify Me</t>
         </is>
       </c>
-      <c r="C364" t="inlineStr">
+      <c r="C364" s="49" t="inlineStr">
         <is>
           <t>Freight DIFOT</t>
         </is>
       </c>
-      <c r="E364" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="F364" t="n">
+      <c r="E364" s="49" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="F364" s="49" t="n">
         <v>48</v>
       </c>
-      <c r="G364" t="n">
+      <c r="G364" s="49" t="n">
         <v>53</v>
       </c>
-      <c r="H364">
+      <c r="H364" s="49">
         <f>F364/G364</f>
         <v/>
       </c>
-      <c r="I364">
+      <c r="I364" s="49">
         <f>IF(H364&gt;=E364,"Yes","No")</f>
         <v/>
       </c>
-      <c r="J364" t="inlineStr">
+      <c r="J364" s="49" t="inlineStr">
         <is>
           <t>Below target - investigate root cause and add to next month's action plan</t>
         </is>
@@ -17685,30 +17685,30 @@
       <c r="A365" s="90" t="n">
         <v>46266</v>
       </c>
-      <c r="B365" t="inlineStr">
+      <c r="B365" s="49" t="inlineStr">
         <is>
           <t>Salt Shark</t>
         </is>
       </c>
-      <c r="C365" t="inlineStr">
+      <c r="C365" s="49" t="inlineStr">
         <is>
           <t>Freight DIFOT</t>
         </is>
       </c>
-      <c r="E365" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="F365" t="n">
+      <c r="E365" s="49" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="F365" s="49" t="n">
         <v>41</v>
       </c>
-      <c r="G365" t="n">
+      <c r="G365" s="49" t="n">
         <v>43</v>
       </c>
-      <c r="H365">
+      <c r="H365" s="49">
         <f>F365/G365</f>
         <v/>
       </c>
-      <c r="I365">
+      <c r="I365" s="49">
         <f>IF(H365&gt;=E365,"Yes","No")</f>
         <v/>
       </c>
@@ -17717,34 +17717,34 @@
       <c r="A366" s="90" t="n">
         <v>46266</v>
       </c>
-      <c r="B366" t="inlineStr">
+      <c r="B366" s="49" t="inlineStr">
         <is>
           <t>Simply Clean</t>
         </is>
       </c>
-      <c r="C366" t="inlineStr">
+      <c r="C366" s="49" t="inlineStr">
         <is>
           <t>Freight DIFOT</t>
         </is>
       </c>
-      <c r="E366" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="F366" t="n">
+      <c r="E366" s="49" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="F366" s="49" t="n">
         <v>87</v>
       </c>
-      <c r="G366" t="n">
+      <c r="G366" s="49" t="n">
         <v>94</v>
       </c>
-      <c r="H366">
+      <c r="H366" s="49">
         <f>F366/G366</f>
         <v/>
       </c>
-      <c r="I366">
+      <c r="I366" s="49">
         <f>IF(H366&gt;=E366,"Yes","No")</f>
         <v/>
       </c>
-      <c r="J366" t="inlineStr">
+      <c r="J366" s="49" t="inlineStr">
         <is>
           <t>Below target - investigate root cause and add to next month's action plan</t>
         </is>
@@ -17754,34 +17754,34 @@
       <c r="A367" s="90" t="n">
         <v>46266</v>
       </c>
-      <c r="B367" t="inlineStr">
+      <c r="B367" s="49" t="inlineStr">
         <is>
           <t>Stryx</t>
         </is>
       </c>
-      <c r="C367" t="inlineStr">
+      <c r="C367" s="49" t="inlineStr">
         <is>
           <t>Freight DIFOT</t>
         </is>
       </c>
-      <c r="E367" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="F367" t="n">
+      <c r="E367" s="49" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="F367" s="49" t="n">
         <v>20</v>
       </c>
-      <c r="G367" t="n">
+      <c r="G367" s="49" t="n">
         <v>22</v>
       </c>
-      <c r="H367">
+      <c r="H367" s="49">
         <f>F367/G367</f>
         <v/>
       </c>
-      <c r="I367">
+      <c r="I367" s="49">
         <f>IF(H367&gt;=E367,"Yes","No")</f>
         <v/>
       </c>
-      <c r="J367" t="inlineStr">
+      <c r="J367" s="49" t="inlineStr">
         <is>
           <t>Below target - investigate root cause and add to next month's action plan</t>
         </is>
@@ -17791,34 +17791,34 @@
       <c r="A368" s="90" t="n">
         <v>46266</v>
       </c>
-      <c r="B368" t="inlineStr">
+      <c r="B368" s="49" t="inlineStr">
         <is>
           <t>Vixxen</t>
         </is>
       </c>
-      <c r="C368" t="inlineStr">
+      <c r="C368" s="49" t="inlineStr">
         <is>
           <t>Freight DIFOT</t>
         </is>
       </c>
-      <c r="E368" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="F368" t="n">
+      <c r="E368" s="49" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="F368" s="49" t="n">
         <v>169</v>
       </c>
-      <c r="G368" t="n">
+      <c r="G368" s="49" t="n">
         <v>185</v>
       </c>
-      <c r="H368">
+      <c r="H368" s="49">
         <f>F368/G368</f>
         <v/>
       </c>
-      <c r="I368">
+      <c r="I368" s="49">
         <f>IF(H368&gt;=E368,"Yes","No")</f>
         <v/>
       </c>
-      <c r="J368" t="inlineStr">
+      <c r="J368" s="49" t="inlineStr">
         <is>
           <t>Below target - investigate root cause and add to next month's action plan</t>
         </is>
@@ -18730,10 +18730,6 @@
         </is>
       </c>
     </row>
-    <row r="36"/>
-    <row r="37"/>
-    <row r="38"/>
-    <row r="39"/>
     <row r="40" ht="15" customHeight="1" s="50">
       <c r="A40" s="77" t="n">
         <v>46196</v>
@@ -20545,32 +20541,32 @@
       <c r="A115" s="90" t="n">
         <v>46303</v>
       </c>
-      <c r="B115" t="inlineStr">
+      <c r="B115" s="49" t="inlineStr">
         <is>
           <t>Oricom</t>
         </is>
       </c>
-      <c r="C115" t="inlineStr">
+      <c r="C115" s="49" t="inlineStr">
         <is>
           <t>HL085007</t>
         </is>
       </c>
-      <c r="D115" t="inlineStr">
+      <c r="D115" s="49" t="inlineStr">
         <is>
           <t>2026-09</t>
         </is>
       </c>
-      <c r="E115" t="inlineStr">
+      <c r="E115" s="49" t="inlineStr">
         <is>
           <t>Freight DIFOT</t>
         </is>
       </c>
-      <c r="F115" t="inlineStr">
+      <c r="F115" s="49" t="inlineStr">
         <is>
           <t>Count as met</t>
         </is>
       </c>
-      <c r="G115" t="inlineStr">
+      <c r="G115" s="49" t="inlineStr">
         <is>
           <t>DC recipient exception - pre-arranged booking, excluded from avg delivery days</t>
         </is>
@@ -20580,32 +20576,32 @@
       <c r="A116" s="90" t="n">
         <v>46303</v>
       </c>
-      <c r="B116" t="inlineStr">
+      <c r="B116" s="49" t="inlineStr">
         <is>
           <t>Oricom</t>
         </is>
       </c>
-      <c r="C116" t="inlineStr">
+      <c r="C116" s="49" t="inlineStr">
         <is>
           <t>4522201808</t>
         </is>
       </c>
-      <c r="D116" t="inlineStr">
+      <c r="D116" s="49" t="inlineStr">
         <is>
           <t>2026-09</t>
         </is>
       </c>
-      <c r="E116" t="inlineStr">
+      <c r="E116" s="49" t="inlineStr">
         <is>
           <t>Freight DIFOT</t>
         </is>
       </c>
-      <c r="F116" t="inlineStr">
+      <c r="F116" s="49" t="inlineStr">
         <is>
           <t>Count as met</t>
         </is>
       </c>
-      <c r="G116" t="inlineStr">
+      <c r="G116" s="49" t="inlineStr">
         <is>
           <t>DC recipient exception - pre-arranged booking, excluded from avg delivery days</t>
         </is>
@@ -20615,32 +20611,32 @@
       <c r="A117" s="90" t="n">
         <v>46303</v>
       </c>
-      <c r="B117" t="inlineStr">
+      <c r="B117" s="49" t="inlineStr">
         <is>
           <t>Oricom</t>
         </is>
       </c>
-      <c r="C117" t="inlineStr">
+      <c r="C117" s="49" t="inlineStr">
         <is>
           <t>4522172931</t>
         </is>
       </c>
-      <c r="D117" t="inlineStr">
+      <c r="D117" s="49" t="inlineStr">
         <is>
           <t>2026-09</t>
         </is>
       </c>
-      <c r="E117" t="inlineStr">
+      <c r="E117" s="49" t="inlineStr">
         <is>
           <t>Freight DIFOT</t>
         </is>
       </c>
-      <c r="F117" t="inlineStr">
+      <c r="F117" s="49" t="inlineStr">
         <is>
           <t>Count as met</t>
         </is>
       </c>
-      <c r="G117" t="inlineStr">
+      <c r="G117" s="49" t="inlineStr">
         <is>
           <t>DC recipient exception - pre-arranged booking, excluded from avg delivery days</t>
         </is>
@@ -20650,32 +20646,32 @@
       <c r="A118" s="90" t="n">
         <v>46303</v>
       </c>
-      <c r="B118" t="inlineStr">
+      <c r="B118" s="49" t="inlineStr">
         <is>
           <t>Oricom</t>
         </is>
       </c>
-      <c r="C118" t="inlineStr">
+      <c r="C118" s="49" t="inlineStr">
         <is>
           <t>4522133734</t>
         </is>
       </c>
-      <c r="D118" t="inlineStr">
+      <c r="D118" s="49" t="inlineStr">
         <is>
           <t>2026-09</t>
         </is>
       </c>
-      <c r="E118" t="inlineStr">
+      <c r="E118" s="49" t="inlineStr">
         <is>
           <t>Freight DIFOT</t>
         </is>
       </c>
-      <c r="F118" t="inlineStr">
+      <c r="F118" s="49" t="inlineStr">
         <is>
           <t>Count as met</t>
         </is>
       </c>
-      <c r="G118" t="inlineStr">
+      <c r="G118" s="49" t="inlineStr">
         <is>
           <t>DC recipient exception - pre-arranged booking, excluded from avg delivery days</t>
         </is>
@@ -20685,32 +20681,32 @@
       <c r="A119" s="90" t="n">
         <v>46303</v>
       </c>
-      <c r="B119" t="inlineStr">
+      <c r="B119" s="49" t="inlineStr">
         <is>
           <t>Oricom</t>
         </is>
       </c>
-      <c r="C119" t="inlineStr">
+      <c r="C119" s="49" t="inlineStr">
         <is>
           <t>4522087338</t>
         </is>
       </c>
-      <c r="D119" t="inlineStr">
+      <c r="D119" s="49" t="inlineStr">
         <is>
           <t>2026-09</t>
         </is>
       </c>
-      <c r="E119" t="inlineStr">
+      <c r="E119" s="49" t="inlineStr">
         <is>
           <t>Freight DIFOT</t>
         </is>
       </c>
-      <c r="F119" t="inlineStr">
+      <c r="F119" s="49" t="inlineStr">
         <is>
           <t>Count as met</t>
         </is>
       </c>
-      <c r="G119" t="inlineStr">
+      <c r="G119" s="49" t="inlineStr">
         <is>
           <t>DC recipient exception - pre-arranged booking, excluded from avg delivery days</t>
         </is>
@@ -20720,32 +20716,32 @@
       <c r="A120" s="90" t="n">
         <v>46303</v>
       </c>
-      <c r="B120" t="inlineStr">
+      <c r="B120" s="49" t="inlineStr">
         <is>
           <t>Oricom</t>
         </is>
       </c>
-      <c r="C120" t="inlineStr">
+      <c r="C120" s="49" t="inlineStr">
         <is>
           <t>4707052687</t>
         </is>
       </c>
-      <c r="D120" t="inlineStr">
+      <c r="D120" s="49" t="inlineStr">
         <is>
           <t>2026-09</t>
         </is>
       </c>
-      <c r="E120" t="inlineStr">
+      <c r="E120" s="49" t="inlineStr">
         <is>
           <t>Freight DIFOT</t>
         </is>
       </c>
-      <c r="F120" t="inlineStr">
+      <c r="F120" s="49" t="inlineStr">
         <is>
           <t>Count as met</t>
         </is>
       </c>
-      <c r="G120" t="inlineStr">
+      <c r="G120" s="49" t="inlineStr">
         <is>
           <t>DC recipient exception - pre-arranged booking, excluded from avg delivery days</t>
         </is>
@@ -21163,7 +21159,6 @@
     <row r="158" ht="15" customHeight="1" s="50">
       <c r="A158" s="83" t="n"/>
     </row>
-    <row r="159"/>
     <row r="160" ht="15" customHeight="1" s="50">
       <c r="A160" s="49" t="inlineStr">
         <is>
@@ -21171,7 +21166,6 @@
         </is>
       </c>
     </row>
-    <row r="161"/>
     <row r="162">
       <c r="A162" s="49" t="inlineStr">
         <is>
@@ -21201,7 +21195,6 @@
         </is>
       </c>
     </row>
-    <row r="165"/>
     <row r="166">
       <c r="A166" s="49" t="inlineStr">
         <is>
@@ -21230,7 +21223,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E15"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="16" customWidth="1" style="49" min="1" max="1"/>
@@ -21488,6 +21481,52 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" s="91" t="n">
+        <v>46309</v>
+      </c>
+      <c r="B14" s="49" t="inlineStr">
+        <is>
+          <t>Coromandel Mountains Company Limited</t>
+        </is>
+      </c>
+      <c r="C14" s="49" t="inlineStr">
+        <is>
+          <t>5311</t>
+        </is>
+      </c>
+      <c r="D14" s="49" t="n">
+        <v>10</v>
+      </c>
+      <c r="E14" s="49" t="inlineStr">
+        <is>
+          <t>Cross-labelled cartons - items shipped with the wrong carton labels</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="91" t="n">
+        <v>46309</v>
+      </c>
+      <c r="B15" s="49" t="inlineStr">
+        <is>
+          <t>Coromandel Mountains Company Limited</t>
+        </is>
+      </c>
+      <c r="C15" s="49" t="inlineStr">
+        <is>
+          <t>5312</t>
+        </is>
+      </c>
+      <c r="D15" s="49" t="n">
+        <v>8</v>
+      </c>
+      <c r="E15" s="49" t="inlineStr">
+        <is>
+          <t>Cross-labelled cartons - items shipped with the wrong carton labels</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A2:E2"/>

</xml_diff>

<commit_message>
Log Made Group NZ Order Cut Off fixed deadline (order 5374), closes #3
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Co-authored-by: Mike-FulfilmentPlus <330614259+Mike-FulfilmentPlus@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/pipeline/kpi_dashboard.xlsx
+++ b/pipeline/kpi_dashboard.xlsx
@@ -17266,30 +17266,30 @@
       <c r="A353" s="90" t="n">
         <v>46266</v>
       </c>
-      <c r="B353" t="inlineStr">
+      <c r="B353" s="49" t="inlineStr">
         <is>
           <t>Aleger Studio</t>
         </is>
       </c>
-      <c r="C353" t="inlineStr">
+      <c r="C353" s="49" t="inlineStr">
         <is>
           <t>Freight DIFOT</t>
         </is>
       </c>
-      <c r="E353" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="F353" t="n">
+      <c r="E353" s="49" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="F353" s="49" t="n">
         <v>6</v>
       </c>
-      <c r="G353" t="n">
+      <c r="G353" s="49" t="n">
         <v>6</v>
       </c>
-      <c r="H353">
+      <c r="H353" s="49">
         <f>F353/G353</f>
         <v/>
       </c>
-      <c r="I353">
+      <c r="I353" s="49">
         <f>IF(H353&gt;=E353,"Yes","No")</f>
         <v/>
       </c>
@@ -17298,34 +17298,34 @@
       <c r="A354" s="90" t="n">
         <v>46266</v>
       </c>
-      <c r="B354" t="inlineStr">
+      <c r="B354" s="49" t="inlineStr">
         <is>
           <t>Coromandel Mountains Company Limited</t>
         </is>
       </c>
-      <c r="C354" t="inlineStr">
+      <c r="C354" s="49" t="inlineStr">
         <is>
           <t>Freight DIFOT</t>
         </is>
       </c>
-      <c r="E354" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="F354" t="n">
+      <c r="E354" s="49" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="F354" s="49" t="n">
         <v>36</v>
       </c>
-      <c r="G354" t="n">
+      <c r="G354" s="49" t="n">
         <v>38</v>
       </c>
-      <c r="H354">
+      <c r="H354" s="49">
         <f>F354/G354</f>
         <v/>
       </c>
-      <c r="I354">
+      <c r="I354" s="49">
         <f>IF(H354&gt;=E354,"Yes","No")</f>
         <v/>
       </c>
-      <c r="J354" t="inlineStr">
+      <c r="J354" s="49" t="inlineStr">
         <is>
           <t>Below target - investigate root cause and add to next month's action plan</t>
         </is>
@@ -17335,34 +17335,34 @@
       <c r="A355" s="90" t="n">
         <v>46266</v>
       </c>
-      <c r="B355" t="inlineStr">
+      <c r="B355" s="49" t="inlineStr">
         <is>
           <t>EcoPallets</t>
         </is>
       </c>
-      <c r="C355" t="inlineStr">
+      <c r="C355" s="49" t="inlineStr">
         <is>
           <t>Freight DIFOT</t>
         </is>
       </c>
-      <c r="E355" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="F355" t="n">
+      <c r="E355" s="49" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="F355" s="49" t="n">
         <v>6</v>
       </c>
-      <c r="G355" t="n">
+      <c r="G355" s="49" t="n">
         <v>7</v>
       </c>
-      <c r="H355">
+      <c r="H355" s="49">
         <f>F355/G355</f>
         <v/>
       </c>
-      <c r="I355">
+      <c r="I355" s="49">
         <f>IF(H355&gt;=E355,"Yes","No")</f>
         <v/>
       </c>
-      <c r="J355" t="inlineStr">
+      <c r="J355" s="49" t="inlineStr">
         <is>
           <t>Below target - investigate root cause and add to next month's action plan</t>
         </is>
@@ -17372,34 +17372,34 @@
       <c r="A356" s="90" t="n">
         <v>46266</v>
       </c>
-      <c r="B356" t="inlineStr">
+      <c r="B356" s="49" t="inlineStr">
         <is>
           <t>Flo &amp; Frankie</t>
         </is>
       </c>
-      <c r="C356" t="inlineStr">
+      <c r="C356" s="49" t="inlineStr">
         <is>
           <t>Freight DIFOT</t>
         </is>
       </c>
-      <c r="E356" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="F356" t="n">
+      <c r="E356" s="49" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="F356" s="49" t="n">
         <v>11</v>
       </c>
-      <c r="G356" t="n">
+      <c r="G356" s="49" t="n">
         <v>13</v>
       </c>
-      <c r="H356">
+      <c r="H356" s="49">
         <f>F356/G356</f>
         <v/>
       </c>
-      <c r="I356">
+      <c r="I356" s="49">
         <f>IF(H356&gt;=E356,"Yes","No")</f>
         <v/>
       </c>
-      <c r="J356" t="inlineStr">
+      <c r="J356" s="49" t="inlineStr">
         <is>
           <t>Below target - investigate root cause and add to next month's action plan</t>
         </is>
@@ -17409,34 +17409,34 @@
       <c r="A357" s="90" t="n">
         <v>46266</v>
       </c>
-      <c r="B357" t="inlineStr">
+      <c r="B357" s="49" t="inlineStr">
         <is>
           <t>Gym Equip</t>
         </is>
       </c>
-      <c r="C357" t="inlineStr">
+      <c r="C357" s="49" t="inlineStr">
         <is>
           <t>Freight DIFOT</t>
         </is>
       </c>
-      <c r="E357" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="F357" t="n">
+      <c r="E357" s="49" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="F357" s="49" t="n">
         <v>17</v>
       </c>
-      <c r="G357" t="n">
+      <c r="G357" s="49" t="n">
         <v>19</v>
       </c>
-      <c r="H357">
+      <c r="H357" s="49">
         <f>F357/G357</f>
         <v/>
       </c>
-      <c r="I357">
+      <c r="I357" s="49">
         <f>IF(H357&gt;=E357,"Yes","No")</f>
         <v/>
       </c>
-      <c r="J357" t="inlineStr">
+      <c r="J357" s="49" t="inlineStr">
         <is>
           <t>Below target - investigate root cause and add to next month's action plan</t>
         </is>
@@ -17446,30 +17446,30 @@
       <c r="A358" s="90" t="n">
         <v>46266</v>
       </c>
-      <c r="B358" t="inlineStr">
+      <c r="B358" s="49" t="inlineStr">
         <is>
           <t>Interior Images</t>
         </is>
       </c>
-      <c r="C358" t="inlineStr">
+      <c r="C358" s="49" t="inlineStr">
         <is>
           <t>Freight DIFOT</t>
         </is>
       </c>
-      <c r="E358" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="F358" t="n">
+      <c r="E358" s="49" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="F358" s="49" t="n">
         <v>1</v>
       </c>
-      <c r="G358" t="n">
+      <c r="G358" s="49" t="n">
         <v>1</v>
       </c>
-      <c r="H358">
+      <c r="H358" s="49">
         <f>F358/G358</f>
         <v/>
       </c>
-      <c r="I358">
+      <c r="I358" s="49">
         <f>IF(H358&gt;=E358,"Yes","No")</f>
         <v/>
       </c>
@@ -17478,34 +17478,34 @@
       <c r="A359" s="90" t="n">
         <v>46266</v>
       </c>
-      <c r="B359" t="inlineStr">
+      <c r="B359" s="49" t="inlineStr">
         <is>
           <t>Jock Freight - SECA</t>
         </is>
       </c>
-      <c r="C359" t="inlineStr">
+      <c r="C359" s="49" t="inlineStr">
         <is>
           <t>Freight DIFOT</t>
         </is>
       </c>
-      <c r="E359" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="F359" t="n">
+      <c r="E359" s="49" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="F359" s="49" t="n">
         <v>8</v>
       </c>
-      <c r="G359" t="n">
+      <c r="G359" s="49" t="n">
         <v>9</v>
       </c>
-      <c r="H359">
+      <c r="H359" s="49">
         <f>F359/G359</f>
         <v/>
       </c>
-      <c r="I359">
+      <c r="I359" s="49">
         <f>IF(H359&gt;=E359,"Yes","No")</f>
         <v/>
       </c>
-      <c r="J359" t="inlineStr">
+      <c r="J359" s="49" t="inlineStr">
         <is>
           <t>Below target - investigate root cause and add to next month's action plan</t>
         </is>
@@ -17515,30 +17515,30 @@
       <c r="A360" s="90" t="n">
         <v>46266</v>
       </c>
-      <c r="B360" t="inlineStr">
+      <c r="B360" s="49" t="inlineStr">
         <is>
           <t>Logwin - Sikla</t>
         </is>
       </c>
-      <c r="C360" t="inlineStr">
+      <c r="C360" s="49" t="inlineStr">
         <is>
           <t>Freight DIFOT</t>
         </is>
       </c>
-      <c r="E360" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="F360" t="n">
+      <c r="E360" s="49" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="F360" s="49" t="n">
         <v>6</v>
       </c>
-      <c r="G360" t="n">
+      <c r="G360" s="49" t="n">
         <v>6</v>
       </c>
-      <c r="H360">
+      <c r="H360" s="49">
         <f>F360/G360</f>
         <v/>
       </c>
-      <c r="I360">
+      <c r="I360" s="49">
         <f>IF(H360&gt;=E360,"Yes","No")</f>
         <v/>
       </c>
@@ -17547,30 +17547,30 @@
       <c r="A361" s="90" t="n">
         <v>46266</v>
       </c>
-      <c r="B361" t="inlineStr">
+      <c r="B361" s="49" t="inlineStr">
         <is>
           <t>Made Group NZ</t>
         </is>
       </c>
-      <c r="C361" t="inlineStr">
+      <c r="C361" s="49" t="inlineStr">
         <is>
           <t>Freight DIFOT</t>
         </is>
       </c>
-      <c r="E361" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="F361" t="n">
+      <c r="E361" s="49" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="F361" s="49" t="n">
         <v>4</v>
       </c>
-      <c r="G361" t="n">
+      <c r="G361" s="49" t="n">
         <v>4</v>
       </c>
-      <c r="H361">
+      <c r="H361" s="49">
         <f>F361/G361</f>
         <v/>
       </c>
-      <c r="I361">
+      <c r="I361" s="49">
         <f>IF(H361&gt;=E361,"Yes","No")</f>
         <v/>
       </c>
@@ -17579,30 +17579,30 @@
       <c r="A362" s="90" t="n">
         <v>46266</v>
       </c>
-      <c r="B362" t="inlineStr">
+      <c r="B362" s="49" t="inlineStr">
         <is>
           <t>May Eleven NZ</t>
         </is>
       </c>
-      <c r="C362" t="inlineStr">
+      <c r="C362" s="49" t="inlineStr">
         <is>
           <t>Freight DIFOT</t>
         </is>
       </c>
-      <c r="E362" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="F362" t="n">
+      <c r="E362" s="49" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="F362" s="49" t="n">
         <v>2</v>
       </c>
-      <c r="G362" t="n">
+      <c r="G362" s="49" t="n">
         <v>2</v>
       </c>
-      <c r="H362">
+      <c r="H362" s="49">
         <f>F362/G362</f>
         <v/>
       </c>
-      <c r="I362">
+      <c r="I362" s="49">
         <f>IF(H362&gt;=E362,"Yes","No")</f>
         <v/>
       </c>
@@ -17611,34 +17611,34 @@
       <c r="A363" s="90" t="n">
         <v>46266</v>
       </c>
-      <c r="B363" t="inlineStr">
+      <c r="B363" s="49" t="inlineStr">
         <is>
           <t>Oricom</t>
         </is>
       </c>
-      <c r="C363" t="inlineStr">
+      <c r="C363" s="49" t="inlineStr">
         <is>
           <t>Freight DIFOT</t>
         </is>
       </c>
-      <c r="E363" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="F363" t="n">
+      <c r="E363" s="49" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="F363" s="49" t="n">
         <v>84</v>
       </c>
-      <c r="G363" t="n">
+      <c r="G363" s="49" t="n">
         <v>91</v>
       </c>
-      <c r="H363">
+      <c r="H363" s="49">
         <f>F363/G363</f>
         <v/>
       </c>
-      <c r="I363">
+      <c r="I363" s="49">
         <f>IF(H363&gt;=E363,"Yes","No")</f>
         <v/>
       </c>
-      <c r="J363" t="inlineStr">
+      <c r="J363" s="49" t="inlineStr">
         <is>
           <t>Below target - investigate root cause and add to next month's action plan</t>
         </is>
@@ -17648,34 +17648,34 @@
       <c r="A364" s="90" t="n">
         <v>46266</v>
       </c>
-      <c r="B364" t="inlineStr">
+      <c r="B364" s="49" t="inlineStr">
         <is>
           <t>Purify Me</t>
         </is>
       </c>
-      <c r="C364" t="inlineStr">
+      <c r="C364" s="49" t="inlineStr">
         <is>
           <t>Freight DIFOT</t>
         </is>
       </c>
-      <c r="E364" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="F364" t="n">
+      <c r="E364" s="49" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="F364" s="49" t="n">
         <v>48</v>
       </c>
-      <c r="G364" t="n">
+      <c r="G364" s="49" t="n">
         <v>53</v>
       </c>
-      <c r="H364">
+      <c r="H364" s="49">
         <f>F364/G364</f>
         <v/>
       </c>
-      <c r="I364">
+      <c r="I364" s="49">
         <f>IF(H364&gt;=E364,"Yes","No")</f>
         <v/>
       </c>
-      <c r="J364" t="inlineStr">
+      <c r="J364" s="49" t="inlineStr">
         <is>
           <t>Below target - investigate root cause and add to next month's action plan</t>
         </is>
@@ -17685,30 +17685,30 @@
       <c r="A365" s="90" t="n">
         <v>46266</v>
       </c>
-      <c r="B365" t="inlineStr">
+      <c r="B365" s="49" t="inlineStr">
         <is>
           <t>Salt Shark</t>
         </is>
       </c>
-      <c r="C365" t="inlineStr">
+      <c r="C365" s="49" t="inlineStr">
         <is>
           <t>Freight DIFOT</t>
         </is>
       </c>
-      <c r="E365" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="F365" t="n">
+      <c r="E365" s="49" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="F365" s="49" t="n">
         <v>41</v>
       </c>
-      <c r="G365" t="n">
+      <c r="G365" s="49" t="n">
         <v>43</v>
       </c>
-      <c r="H365">
+      <c r="H365" s="49">
         <f>F365/G365</f>
         <v/>
       </c>
-      <c r="I365">
+      <c r="I365" s="49">
         <f>IF(H365&gt;=E365,"Yes","No")</f>
         <v/>
       </c>
@@ -17717,34 +17717,34 @@
       <c r="A366" s="90" t="n">
         <v>46266</v>
       </c>
-      <c r="B366" t="inlineStr">
+      <c r="B366" s="49" t="inlineStr">
         <is>
           <t>Simply Clean</t>
         </is>
       </c>
-      <c r="C366" t="inlineStr">
+      <c r="C366" s="49" t="inlineStr">
         <is>
           <t>Freight DIFOT</t>
         </is>
       </c>
-      <c r="E366" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="F366" t="n">
+      <c r="E366" s="49" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="F366" s="49" t="n">
         <v>87</v>
       </c>
-      <c r="G366" t="n">
+      <c r="G366" s="49" t="n">
         <v>94</v>
       </c>
-      <c r="H366">
+      <c r="H366" s="49">
         <f>F366/G366</f>
         <v/>
       </c>
-      <c r="I366">
+      <c r="I366" s="49">
         <f>IF(H366&gt;=E366,"Yes","No")</f>
         <v/>
       </c>
-      <c r="J366" t="inlineStr">
+      <c r="J366" s="49" t="inlineStr">
         <is>
           <t>Below target - investigate root cause and add to next month's action plan</t>
         </is>
@@ -17754,34 +17754,34 @@
       <c r="A367" s="90" t="n">
         <v>46266</v>
       </c>
-      <c r="B367" t="inlineStr">
+      <c r="B367" s="49" t="inlineStr">
         <is>
           <t>Stryx</t>
         </is>
       </c>
-      <c r="C367" t="inlineStr">
+      <c r="C367" s="49" t="inlineStr">
         <is>
           <t>Freight DIFOT</t>
         </is>
       </c>
-      <c r="E367" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="F367" t="n">
+      <c r="E367" s="49" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="F367" s="49" t="n">
         <v>20</v>
       </c>
-      <c r="G367" t="n">
+      <c r="G367" s="49" t="n">
         <v>22</v>
       </c>
-      <c r="H367">
+      <c r="H367" s="49">
         <f>F367/G367</f>
         <v/>
       </c>
-      <c r="I367">
+      <c r="I367" s="49">
         <f>IF(H367&gt;=E367,"Yes","No")</f>
         <v/>
       </c>
-      <c r="J367" t="inlineStr">
+      <c r="J367" s="49" t="inlineStr">
         <is>
           <t>Below target - investigate root cause and add to next month's action plan</t>
         </is>
@@ -17791,34 +17791,34 @@
       <c r="A368" s="90" t="n">
         <v>46266</v>
       </c>
-      <c r="B368" t="inlineStr">
+      <c r="B368" s="49" t="inlineStr">
         <is>
           <t>Vixxen</t>
         </is>
       </c>
-      <c r="C368" t="inlineStr">
+      <c r="C368" s="49" t="inlineStr">
         <is>
           <t>Freight DIFOT</t>
         </is>
       </c>
-      <c r="E368" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="F368" t="n">
+      <c r="E368" s="49" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="F368" s="49" t="n">
         <v>169</v>
       </c>
-      <c r="G368" t="n">
+      <c r="G368" s="49" t="n">
         <v>185</v>
       </c>
-      <c r="H368">
+      <c r="H368" s="49">
         <f>F368/G368</f>
         <v/>
       </c>
-      <c r="I368">
+      <c r="I368" s="49">
         <f>IF(H368&gt;=E368,"Yes","No")</f>
         <v/>
       </c>
-      <c r="J368" t="inlineStr">
+      <c r="J368" s="49" t="inlineStr">
         <is>
           <t>Below target - investigate root cause and add to next month's action plan</t>
         </is>
@@ -18730,10 +18730,6 @@
         </is>
       </c>
     </row>
-    <row r="36"/>
-    <row r="37"/>
-    <row r="38"/>
-    <row r="39"/>
     <row r="40" ht="15" customHeight="1" s="50">
       <c r="A40" s="77" t="n">
         <v>46196</v>
@@ -20545,32 +20541,32 @@
       <c r="A115" s="90" t="n">
         <v>46303</v>
       </c>
-      <c r="B115" t="inlineStr">
+      <c r="B115" s="49" t="inlineStr">
         <is>
           <t>Oricom</t>
         </is>
       </c>
-      <c r="C115" t="inlineStr">
+      <c r="C115" s="49" t="inlineStr">
         <is>
           <t>HL085007</t>
         </is>
       </c>
-      <c r="D115" t="inlineStr">
+      <c r="D115" s="49" t="inlineStr">
         <is>
           <t>2026-09</t>
         </is>
       </c>
-      <c r="E115" t="inlineStr">
+      <c r="E115" s="49" t="inlineStr">
         <is>
           <t>Freight DIFOT</t>
         </is>
       </c>
-      <c r="F115" t="inlineStr">
+      <c r="F115" s="49" t="inlineStr">
         <is>
           <t>Count as met</t>
         </is>
       </c>
-      <c r="G115" t="inlineStr">
+      <c r="G115" s="49" t="inlineStr">
         <is>
           <t>DC recipient exception - pre-arranged booking, excluded from avg delivery days</t>
         </is>
@@ -20580,32 +20576,32 @@
       <c r="A116" s="90" t="n">
         <v>46303</v>
       </c>
-      <c r="B116" t="inlineStr">
+      <c r="B116" s="49" t="inlineStr">
         <is>
           <t>Oricom</t>
         </is>
       </c>
-      <c r="C116" t="inlineStr">
+      <c r="C116" s="49" t="inlineStr">
         <is>
           <t>4522201808</t>
         </is>
       </c>
-      <c r="D116" t="inlineStr">
+      <c r="D116" s="49" t="inlineStr">
         <is>
           <t>2026-09</t>
         </is>
       </c>
-      <c r="E116" t="inlineStr">
+      <c r="E116" s="49" t="inlineStr">
         <is>
           <t>Freight DIFOT</t>
         </is>
       </c>
-      <c r="F116" t="inlineStr">
+      <c r="F116" s="49" t="inlineStr">
         <is>
           <t>Count as met</t>
         </is>
       </c>
-      <c r="G116" t="inlineStr">
+      <c r="G116" s="49" t="inlineStr">
         <is>
           <t>DC recipient exception - pre-arranged booking, excluded from avg delivery days</t>
         </is>
@@ -20615,32 +20611,32 @@
       <c r="A117" s="90" t="n">
         <v>46303</v>
       </c>
-      <c r="B117" t="inlineStr">
+      <c r="B117" s="49" t="inlineStr">
         <is>
           <t>Oricom</t>
         </is>
       </c>
-      <c r="C117" t="inlineStr">
+      <c r="C117" s="49" t="inlineStr">
         <is>
           <t>4522172931</t>
         </is>
       </c>
-      <c r="D117" t="inlineStr">
+      <c r="D117" s="49" t="inlineStr">
         <is>
           <t>2026-09</t>
         </is>
       </c>
-      <c r="E117" t="inlineStr">
+      <c r="E117" s="49" t="inlineStr">
         <is>
           <t>Freight DIFOT</t>
         </is>
       </c>
-      <c r="F117" t="inlineStr">
+      <c r="F117" s="49" t="inlineStr">
         <is>
           <t>Count as met</t>
         </is>
       </c>
-      <c r="G117" t="inlineStr">
+      <c r="G117" s="49" t="inlineStr">
         <is>
           <t>DC recipient exception - pre-arranged booking, excluded from avg delivery days</t>
         </is>
@@ -20650,32 +20646,32 @@
       <c r="A118" s="90" t="n">
         <v>46303</v>
       </c>
-      <c r="B118" t="inlineStr">
+      <c r="B118" s="49" t="inlineStr">
         <is>
           <t>Oricom</t>
         </is>
       </c>
-      <c r="C118" t="inlineStr">
+      <c r="C118" s="49" t="inlineStr">
         <is>
           <t>4522133734</t>
         </is>
       </c>
-      <c r="D118" t="inlineStr">
+      <c r="D118" s="49" t="inlineStr">
         <is>
           <t>2026-09</t>
         </is>
       </c>
-      <c r="E118" t="inlineStr">
+      <c r="E118" s="49" t="inlineStr">
         <is>
           <t>Freight DIFOT</t>
         </is>
       </c>
-      <c r="F118" t="inlineStr">
+      <c r="F118" s="49" t="inlineStr">
         <is>
           <t>Count as met</t>
         </is>
       </c>
-      <c r="G118" t="inlineStr">
+      <c r="G118" s="49" t="inlineStr">
         <is>
           <t>DC recipient exception - pre-arranged booking, excluded from avg delivery days</t>
         </is>
@@ -20685,32 +20681,32 @@
       <c r="A119" s="90" t="n">
         <v>46303</v>
       </c>
-      <c r="B119" t="inlineStr">
+      <c r="B119" s="49" t="inlineStr">
         <is>
           <t>Oricom</t>
         </is>
       </c>
-      <c r="C119" t="inlineStr">
+      <c r="C119" s="49" t="inlineStr">
         <is>
           <t>4522087338</t>
         </is>
       </c>
-      <c r="D119" t="inlineStr">
+      <c r="D119" s="49" t="inlineStr">
         <is>
           <t>2026-09</t>
         </is>
       </c>
-      <c r="E119" t="inlineStr">
+      <c r="E119" s="49" t="inlineStr">
         <is>
           <t>Freight DIFOT</t>
         </is>
       </c>
-      <c r="F119" t="inlineStr">
+      <c r="F119" s="49" t="inlineStr">
         <is>
           <t>Count as met</t>
         </is>
       </c>
-      <c r="G119" t="inlineStr">
+      <c r="G119" s="49" t="inlineStr">
         <is>
           <t>DC recipient exception - pre-arranged booking, excluded from avg delivery days</t>
         </is>
@@ -20720,32 +20716,32 @@
       <c r="A120" s="90" t="n">
         <v>46303</v>
       </c>
-      <c r="B120" t="inlineStr">
+      <c r="B120" s="49" t="inlineStr">
         <is>
           <t>Oricom</t>
         </is>
       </c>
-      <c r="C120" t="inlineStr">
+      <c r="C120" s="49" t="inlineStr">
         <is>
           <t>4707052687</t>
         </is>
       </c>
-      <c r="D120" t="inlineStr">
+      <c r="D120" s="49" t="inlineStr">
         <is>
           <t>2026-09</t>
         </is>
       </c>
-      <c r="E120" t="inlineStr">
+      <c r="E120" s="49" t="inlineStr">
         <is>
           <t>Freight DIFOT</t>
         </is>
       </c>
-      <c r="F120" t="inlineStr">
+      <c r="F120" s="49" t="inlineStr">
         <is>
           <t>Count as met</t>
         </is>
       </c>
-      <c r="G120" t="inlineStr">
+      <c r="G120" s="49" t="inlineStr">
         <is>
           <t>DC recipient exception - pre-arranged booking, excluded from avg delivery days</t>
         </is>
@@ -20927,7 +20923,34 @@
         <v>46300</v>
       </c>
     </row>
-    <row r="131" ht="23.85" customHeight="1" s="50"/>
+    <row r="131" ht="23.85" customHeight="1" s="50">
+      <c r="A131" s="49" t="inlineStr">
+        <is>
+          <t>Made Group NZ</t>
+        </is>
+      </c>
+      <c r="B131" s="49" t="inlineStr">
+        <is>
+          <t>All Orders</t>
+        </is>
+      </c>
+      <c r="C131" s="49" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="D131" s="49" t="inlineStr">
+        <is>
+          <t>Fixed (2026-10-16 13:00)</t>
+        </is>
+      </c>
+      <c r="E131" s="83" t="n">
+        <v>46309</v>
+      </c>
+      <c r="F131" s="83" t="n">
+        <v>46309</v>
+      </c>
+    </row>
     <row r="132" ht="15" customHeight="1" s="50"/>
     <row r="133" ht="15" customHeight="1" s="50"/>
     <row r="134" ht="23.85" customHeight="1" s="50"/>
@@ -21163,7 +21186,6 @@
     <row r="158" ht="15" customHeight="1" s="50">
       <c r="A158" s="83" t="n"/>
     </row>
-    <row r="159"/>
     <row r="160" ht="15" customHeight="1" s="50">
       <c r="A160" s="49" t="inlineStr">
         <is>
@@ -21171,7 +21193,6 @@
         </is>
       </c>
     </row>
-    <row r="161"/>
     <row r="162">
       <c r="A162" s="49" t="inlineStr">
         <is>
@@ -21201,7 +21222,6 @@
         </is>
       </c>
     </row>
-    <row r="165"/>
     <row r="166">
       <c r="A166" s="49" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Log Coromandel Mountains cross-labelled cartons 5311 and 5312
Co-authored-by: Mike-FulfilmentPlus <330614259+Mike-FulfilmentPlus@users.noreply.github.com>

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/pipeline/kpi_dashboard.xlsx
+++ b/pipeline/kpi_dashboard.xlsx
@@ -21230,7 +21230,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E15"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="16" customWidth="1" style="49" min="1" max="1"/>
@@ -21488,6 +21488,52 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" s="91" t="n">
+        <v>46309</v>
+      </c>
+      <c r="B14" s="49" t="inlineStr">
+        <is>
+          <t>Coromandel Mountains Company Limited</t>
+        </is>
+      </c>
+      <c r="C14" s="49" t="inlineStr">
+        <is>
+          <t>5311</t>
+        </is>
+      </c>
+      <c r="D14" s="49" t="n">
+        <v>10</v>
+      </c>
+      <c r="E14" s="49" t="inlineStr">
+        <is>
+          <t>Cross-labelled cartons</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="91" t="n">
+        <v>46309</v>
+      </c>
+      <c r="B15" s="49" t="inlineStr">
+        <is>
+          <t>Coromandel Mountains Company Limited</t>
+        </is>
+      </c>
+      <c r="C15" s="49" t="inlineStr">
+        <is>
+          <t>5312</t>
+        </is>
+      </c>
+      <c r="D15" s="49" t="n">
+        <v>8</v>
+      </c>
+      <c r="E15" s="49" t="inlineStr">
+        <is>
+          <t>Cross-labelled cartons</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A2:E2"/>

</xml_diff>

<commit_message>
Log from issue #2 (catch-up merge)
</commit_message>
<xml_diff>
--- a/pipeline/kpi_dashboard.xlsx
+++ b/pipeline/kpi_dashboard.xlsx
@@ -21230,7 +21230,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E15"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="16" customWidth="1" style="49" min="1" max="1"/>
@@ -21488,6 +21488,52 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" s="91" t="n">
+        <v>46310</v>
+      </c>
+      <c r="B14" s="49" t="inlineStr">
+        <is>
+          <t>Coromandel Mountains Company Limited</t>
+        </is>
+      </c>
+      <c r="C14" s="49" t="inlineStr">
+        <is>
+          <t>5311</t>
+        </is>
+      </c>
+      <c r="D14" s="49" t="n">
+        <v>10</v>
+      </c>
+      <c r="E14" s="49" t="inlineStr">
+        <is>
+          <t>Cross-labelled cartons</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="91" t="n">
+        <v>46310</v>
+      </c>
+      <c r="B15" s="49" t="inlineStr">
+        <is>
+          <t>Coromandel Mountains Company Limited</t>
+        </is>
+      </c>
+      <c r="C15" s="49" t="inlineStr">
+        <is>
+          <t>5312</t>
+        </is>
+      </c>
+      <c r="D15" s="49" t="n">
+        <v>8</v>
+      </c>
+      <c r="E15" s="49" t="inlineStr">
+        <is>
+          <t>Cross-labelled cartons</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A2:E2"/>

</xml_diff>